<commit_message>
Replace USB-first POPS UDPFS with network read/write Assault 1.0.0
Preserve the UDPFS mode key, migrate stale Alpha pairs by byte verification, use MC SYS-CONF precedence, and package matching release drivers and notices. Add real-Lua configuration and production-launch regressions.

Co-authored-by: ChatGPT <chatgpt@openai.com>
</commit_message>
<xml_diff>
--- a/docs/translations/slovak.xlsx
+++ b/docs/translations/slovak.xlsx
@@ -133,8 +133,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SlovakTranslations" displayName="SlovakTranslations" ref="A7:D415" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:D415"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SlovakTranslations" displayName="SlovakTranslations" ref="A7:D416" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:D416"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="English (do not edit)"/>
     <x:tableColumn id="2" name="Slovak (put your translation here)"/>
@@ -337,7 +337,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
     <x:tabColor rgb="FF243D5A"/>
   </x:sheetPr>
@@ -365,7 +365,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>408 English strings. Enter Slovak in the yellow cells in column B.</x:v>
+        <x:v>409 English strings. Enter Slovak in the yellow cells in column B.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -488,7 +488,7 @@
       <x:c r="B15" s="7" t="str"/>
       <x:c r="C15" s="5" t="str"/>
       <x:c r="D15" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:7272</x:v>
+        <x:v>bin/POPSLDR/system.lua:7285</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
@@ -500,7 +500,7 @@
         <x:v>Keep in order: %s; Keep literal \n line breaks</x:v>
       </x:c>
       <x:c r="D16" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10552</x:v>
+        <x:v>bin/POPSLDR/system.lua:10583</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="46" customHeight="1">
@@ -598,7 +598,7 @@
       <x:c r="B25" s="7" t="str"/>
       <x:c r="C25" s="5" t="str"/>
       <x:c r="D25" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:7272</x:v>
+        <x:v>bin/POPSLDR/system.lua:7285</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="46" customHeight="1">
@@ -670,7 +670,7 @@
         <x:v>Keep in order: %s</x:v>
       </x:c>
       <x:c r="D32" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10560</x:v>
+        <x:v>bin/POPSLDR/system.lua:10591</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="46" customHeight="1">
@@ -682,7 +682,7 @@
         <x:v>Keep in order: %s</x:v>
       </x:c>
       <x:c r="D33" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10503</x:v>
+        <x:v>bin/POPSLDR/system.lua:10534</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="46" customHeight="1">
@@ -734,7 +734,7 @@
       <x:c r="B38" s="7" t="str"/>
       <x:c r="C38" s="5" t="str"/>
       <x:c r="D38" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:7129; bin/POPSLDR/system.lua:7691</x:v>
+        <x:v>bin/POPSLDR/system.lua:7134; bin/POPSLDR/system.lua:7704</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="46" customHeight="1">
@@ -798,7 +798,7 @@
         <x:v>Keep literal \n line breaks</x:v>
       </x:c>
       <x:c r="D44" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10739</x:v>
+        <x:v>bin/POPSLDR/system.lua:10770</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="46" customHeight="1">
@@ -936,7 +936,7 @@
       <x:c r="B57" s="7" t="str"/>
       <x:c r="C57" s="5" t="str"/>
       <x:c r="D57" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:5391; bin/POPSLDR/system.lua:7065; bin/POPSLDR/system.lua:7446</x:v>
+        <x:v>bin/POPSLDR/system.lua:5391; bin/POPSLDR/system.lua:7065; bin/POPSLDR/system.lua:7459</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="46" customHeight="1">
@@ -946,7 +946,7 @@
       <x:c r="B58" s="7" t="str"/>
       <x:c r="C58" s="5" t="str"/>
       <x:c r="D58" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8214</x:v>
+        <x:v>bin/POPSLDR/system.lua:8227</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="46" customHeight="1">
@@ -966,7 +966,7 @@
       <x:c r="B60" s="7" t="str"/>
       <x:c r="C60" s="5" t="str"/>
       <x:c r="D60" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8240</x:v>
+        <x:v>bin/POPSLDR/system.lua:8253</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="46" customHeight="1">
@@ -1016,7 +1016,7 @@
       <x:c r="B65" s="7" t="str"/>
       <x:c r="C65" s="5" t="str"/>
       <x:c r="D65" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10150</x:v>
+        <x:v>bin/POPSLDR/system.lua:10181</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="46" customHeight="1">
@@ -1153,7 +1153,7 @@
     </x:row>
     <x:row r="79" ht="46" customHeight="1">
       <x:c r="A79" s="6" t="str">
-        <x:v>Could not open USB+UDPFS</x:v>
+        <x:v>Could not open UDPFS</x:v>
       </x:c>
       <x:c r="B79" s="7" t="str"/>
       <x:c r="C79" s="5" t="str"/>
@@ -1168,83 +1168,83 @@
       <x:c r="B80" s="7" t="str"/>
       <x:c r="C80" s="5" t="str"/>
       <x:c r="D80" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10494</x:v>
+        <x:v>bin/POPSLDR/system.lua:10525</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="46" customHeight="1">
       <x:c r="A81" s="6" t="str">
-        <x:v>Could not start MX4SIO</x:v>
+        <x:v>Could not read UDPFS configuration:\n%s</x:v>
       </x:c>
       <x:c r="B81" s="7" t="str"/>
-      <x:c r="C81" s="5" t="str"/>
+      <x:c r="C81" s="5" t="str">
+        <x:v>Keep in order: %s</x:v>
+      </x:c>
       <x:c r="D81" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6087</x:v>
+        <x:v>bin/POPSLDR/system.lua:8467</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="46" customHeight="1">
       <x:c r="A82" s="6" t="str">
-        <x:v>Could not start the internal drive</x:v>
+        <x:v>Could not start MX4SIO</x:v>
       </x:c>
       <x:c r="B82" s="7" t="str"/>
       <x:c r="C82" s="5" t="str"/>
       <x:c r="D82" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10458; bin/POPSLDR/ui.lua:6147</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6087</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="46" customHeight="1">
       <x:c r="A83" s="6" t="str">
-        <x:v>Could not write UDPFS configuration:\n%s</x:v>
+        <x:v>Could not start the internal drive</x:v>
       </x:c>
       <x:c r="B83" s="7" t="str"/>
-      <x:c r="C83" s="5" t="str">
-        <x:v>Keep in order: %s; Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C83" s="5" t="str"/>
       <x:c r="D83" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8444</x:v>
+        <x:v>bin/POPSLDR/system.lua:10489; bin/POPSLDR/ui.lua:6147</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="46" customHeight="1">
       <x:c r="A84" s="6" t="str">
-        <x:v>Couldn't apply the PS2 IP settings\ntry again or power-cycle the network adapter</x:v>
+        <x:v>Could not write UDPFS configuration:\n%s</x:v>
       </x:c>
       <x:c r="B84" s="7" t="str"/>
       <x:c r="C84" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
+        <x:v>Keep in order: %s; Keep literal \n line breaks</x:v>
       </x:c>
       <x:c r="D84" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6919</x:v>
+        <x:v>bin/POPSLDR/system.lua:8475</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="46" customHeight="1">
       <x:c r="A85" s="6" t="str">
-        <x:v>Couldn't read that game selection</x:v>
+        <x:v>Couldn't apply the PS2 IP settings\ntry again or power-cycle the network adapter</x:v>
       </x:c>
       <x:c r="B85" s="7" t="str"/>
-      <x:c r="C85" s="5" t="str"/>
+      <x:c r="C85" s="5" t="str">
+        <x:v>Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D85" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3679</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6919</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="46" customHeight="1">
       <x:c r="A86" s="6" t="str">
-        <x:v>Couldn't restore BDMA mode</x:v>
+        <x:v>Couldn't read that game selection</x:v>
       </x:c>
       <x:c r="B86" s="7" t="str"/>
       <x:c r="C86" s="5" t="str"/>
       <x:c r="D86" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:5929</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3679</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="46" customHeight="1">
       <x:c r="A87" s="6" t="str">
-        <x:v>Couldn't save settings\n%s may be read-only</x:v>
+        <x:v>Couldn't restore BDMA mode</x:v>
       </x:c>
       <x:c r="B87" s="7" t="str"/>
-      <x:c r="C87" s="5" t="str">
-        <x:v>Keep in order: %s; Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C87" s="5" t="str"/>
       <x:c r="D87" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4556</x:v>
+        <x:v>bin/POPSLDR/system.lua:5929</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="46" customHeight="1">
@@ -1269,1518 +1269,1518 @@
     </x:row>
     <x:row r="90" ht="46" customHeight="1">
       <x:c r="A90" s="6" t="str">
-        <x:v>Couldn't update hidden state</x:v>
+        <x:v>Couldn't save settings\n%s may be read-only</x:v>
       </x:c>
       <x:c r="B90" s="7" t="str"/>
-      <x:c r="C90" s="5" t="str"/>
+      <x:c r="C90" s="5" t="str">
+        <x:v>Keep in order: %s; Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D90" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4203</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4556</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="46" customHeight="1">
       <x:c r="A91" s="6" t="str">
-        <x:v>Couldn't write %s</x:v>
+        <x:v>Couldn't update hidden state</x:v>
       </x:c>
       <x:c r="B91" s="7" t="str"/>
-      <x:c r="C91" s="5" t="str">
-        <x:v>Keep in order: %s</x:v>
-      </x:c>
+      <x:c r="C91" s="5" t="str"/>
       <x:c r="D91" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3904</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4203</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="46" customHeight="1">
       <x:c r="A92" s="6" t="str">
-        <x:v>Couldn't write .hide to the HDD</x:v>
+        <x:v>Couldn't write %s</x:v>
       </x:c>
       <x:c r="B92" s="7" t="str"/>
-      <x:c r="C92" s="5" t="str"/>
+      <x:c r="C92" s="5" t="str">
+        <x:v>Keep in order: %s</x:v>
+      </x:c>
       <x:c r="D92" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4167</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3904</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="46" customHeight="1">
       <x:c r="A93" s="6" t="str">
-        <x:v>Cover art</x:v>
+        <x:v>Couldn't write .hide to the HDD</x:v>
       </x:c>
       <x:c r="B93" s="7" t="str"/>
       <x:c r="C93" s="5" t="str"/>
       <x:c r="D93" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5108</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4167</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="46" customHeight="1">
       <x:c r="A94" s="6" t="str">
-        <x:v>Credits</x:v>
+        <x:v>Cover art</x:v>
       </x:c>
       <x:c r="B94" s="7" t="str"/>
       <x:c r="C94" s="5" t="str"/>
       <x:c r="D94" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5375</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5108</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="46" customHeight="1">
       <x:c r="A95" s="6" t="str">
-        <x:v>Cursor: L1 / R1</x:v>
+        <x:v>Credits</x:v>
       </x:c>
       <x:c r="B95" s="7" t="str"/>
       <x:c r="C95" s="5" t="str"/>
       <x:c r="D95" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:2828</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5375</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="46" customHeight="1">
       <x:c r="A96" s="6" t="str">
-        <x:v>DEL</x:v>
+        <x:v>Cursor: L1 / R1</x:v>
       </x:c>
       <x:c r="B96" s="7" t="str"/>
       <x:c r="C96" s="5" t="str"/>
       <x:c r="D96" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:2429; bin/POPSLDR/ui.lua:2439; bin/POPSLDR/ui.lua:2451</x:v>
+        <x:v>bin/POPSLDR/ui.lua:2828</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="46" customHeight="1">
       <x:c r="A97" s="6" t="str">
-        <x:v>DEV9 module failed to load</x:v>
+        <x:v>DEL</x:v>
       </x:c>
       <x:c r="B97" s="7" t="str"/>
       <x:c r="C97" s="5" t="str"/>
       <x:c r="D97" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6935</x:v>
+        <x:v>bin/POPSLDR/ui.lua:2429; bin/POPSLDR/ui.lua:2439; bin/POPSLDR/ui.lua:2451</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="46" customHeight="1">
       <x:c r="A98" s="6" t="str">
-        <x:v>DHCP (automatic)</x:v>
+        <x:v>DEV9 module failed to load</x:v>
       </x:c>
       <x:c r="B98" s="7" t="str"/>
       <x:c r="C98" s="5" t="str"/>
       <x:c r="D98" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7250</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6935</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="46" customHeight="1">
       <x:c r="A99" s="6" t="str">
-        <x:v>DHCP failed\nset a static IP in SMB settings</x:v>
+        <x:v>DHCP (automatic)</x:v>
       </x:c>
       <x:c r="B99" s="7" t="str"/>
-      <x:c r="C99" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C99" s="5" t="str"/>
       <x:c r="D99" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6920</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7250</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="46" customHeight="1">
       <x:c r="A100" s="6" t="str">
-        <x:v>DKWDRV Path</x:v>
+        <x:v>DHCP failed\nset a static IP in SMB settings</x:v>
       </x:c>
       <x:c r="B100" s="7" t="str"/>
-      <x:c r="C100" s="5" t="str"/>
+      <x:c r="C100" s="5" t="str">
+        <x:v>Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D100" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5249</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6920</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="46" customHeight="1">
       <x:c r="A101" s="6" t="str">
-        <x:v>DKWDRV failed to launch</x:v>
+        <x:v>DKWDRV Path</x:v>
       </x:c>
       <x:c r="B101" s="7" t="str"/>
       <x:c r="C101" s="5" t="str"/>
       <x:c r="D101" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:2205</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5249</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="46" customHeight="1">
       <x:c r="A102" s="6" t="str">
-        <x:v>DNS</x:v>
+        <x:v>DKWDRV failed to launch</x:v>
       </x:c>
       <x:c r="B102" s="7" t="str"/>
       <x:c r="C102" s="5" t="str"/>
       <x:c r="D102" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:4995; bin/POPSLDR/system.lua:5047; bin/POPSLDR/ui.lua:7211</x:v>
+        <x:v>bin/POPSLDR/ui.lua:2205</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="46" customHeight="1">
       <x:c r="A103" s="6" t="str">
-        <x:v>DONE</x:v>
+        <x:v>DNS</x:v>
       </x:c>
       <x:c r="B103" s="7" t="str"/>
       <x:c r="C103" s="5" t="str"/>
       <x:c r="D103" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:2430; bin/POPSLDR/ui.lua:2440; bin/POPSLDR/ui.lua:2452</x:v>
+        <x:v>bin/POPSLDR/system.lua:4995; bin/POPSLDR/system.lua:5047; bin/POPSLDR/ui.lua:7211</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="46" customHeight="1">
       <x:c r="A104" s="6" t="str">
-        <x:v>Default</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="B104" s="7" t="str"/>
-      <x:c r="C104" s="5" t="str">
-        <x:v>Ember: Unchanged preserves a setting; Default removes the override</x:v>
-      </x:c>
+      <x:c r="C104" s="5" t="str"/>
       <x:c r="D104" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5219</x:v>
+        <x:v>bin/POPSLDR/ui.lua:2430; bin/POPSLDR/ui.lua:2440; bin/POPSLDR/ui.lua:2452</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="46" customHeight="1">
       <x:c r="A105" s="6" t="str">
-        <x:v>Default (global)</x:v>
+        <x:v>Default</x:v>
       </x:c>
       <x:c r="B105" s="7" t="str"/>
       <x:c r="C105" s="5" t="str">
         <x:v>Ember: Unchanged preserves a setting; Default removes the override</x:v>
       </x:c>
       <x:c r="D105" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3889</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5219</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="46" customHeight="1">
       <x:c r="A106" s="6" t="str">
-        <x:v>Defaults restored</x:v>
+        <x:v>Default (global)</x:v>
       </x:c>
       <x:c r="B106" s="7" t="str"/>
-      <x:c r="C106" s="5" t="str"/>
+      <x:c r="C106" s="5" t="str">
+        <x:v>Ember: Unchanged preserves a setting; Default removes the override</x:v>
+      </x:c>
       <x:c r="D106" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4758</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3889</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="46" customHeight="1">
       <x:c r="A107" s="6" t="str">
-        <x:v>Delete the POPSTARTER folder from the memory card?</x:v>
+        <x:v>Defaults restored</x:v>
       </x:c>
       <x:c r="B107" s="7" t="str"/>
       <x:c r="C107" s="5" t="str"/>
       <x:c r="D107" s="5" t="str">
+        <x:v>bin/POPSLDR/ui.lua:4758</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="46" customHeight="1">
+      <x:c r="A108" s="6" t="str">
+        <x:v>Delete the POPSTARTER folder from the memory card?</x:v>
+      </x:c>
+      <x:c r="B108" s="7" t="str"/>
+      <x:c r="C108" s="5" t="str"/>
+      <x:c r="D108" s="5" t="str">
         <x:v>bin/POPSLDR/ui.lua:5326</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="108" ht="112" customHeight="1">
-      <x:c r="A108" s="6" t="str">
-        <x:v>Design by Berion\nScripts by nuno6573 and Ripto\nBased on Enceladus by Daniel Santos\nTesting by P4NCHOL1NO, VizoR, provato,\nnuno6573, oldman63, saildot4k, and Community\n\nSpecial Thanks To:\nkrHACKen for making POPStarter\nuyjulian, fjtrujy, HWC, and others for always helping\n\nThis program is free and open source\nIf you bought it, you have been scammed\n\nCompatibility problems? Visit:\nyoutube.com/@hugopocked6695</x:v>
-      </x:c>
-      <x:c r="B108" s="7" t="str"/>
-      <x:c r="C108" s="5" t="str">
-        <x:v>Keep literal \n line breaks; Credits: keep names, handles and URL unchanged</x:v>
-      </x:c>
-      <x:c r="D108" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6566</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="46" customHeight="1">
       <x:c r="A109" s="6" t="str">
-        <x:v>Detecting MMCE device...</x:v>
+        <x:v>Design by Berion\nScripts by nuno6573 and Ripto\nBased on Enceladus by Daniel Santos\nTesting by P4NCHOL1NO, VizoR, provato,\nnuno6573, oldman63, saildot4k, and Community\n\nSpecial Thanks To:\nkrHACKen for making POPStarter\nuyjulian, fjtrujy, HWC, and others for always helping\n\nThis program is free and open source\nIf you bought it, you have been scammed\n\nCompatibility problems? Visit:\nyoutube.com/@hugopocked6695</x:v>
       </x:c>
       <x:c r="B109" s="7" t="str"/>
-      <x:c r="C109" s="5" t="str"/>
+      <x:c r="C109" s="5" t="str">
+        <x:v>Keep literal \n line breaks; Credits: keep names, handles and URL unchanged</x:v>
+      </x:c>
       <x:c r="D109" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4041; bin/POPSLDR/ui.lua:6021</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6566</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="46" customHeight="1">
       <x:c r="A110" s="6" t="str">
-        <x:v>Device List</x:v>
+        <x:v>Detecting MMCE device...</x:v>
       </x:c>
       <x:c r="B110" s="7" t="str"/>
       <x:c r="C110" s="5" t="str"/>
       <x:c r="D110" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4998</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4041; bin/POPSLDR/ui.lua:6021</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="46" customHeight="1">
       <x:c r="A111" s="6" t="str">
-        <x:v>Disabled</x:v>
+        <x:v>Device List</x:v>
       </x:c>
       <x:c r="B111" s="7" t="str"/>
       <x:c r="C111" s="5" t="str"/>
       <x:c r="D111" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5044</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4998</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="46" customHeight="1">
       <x:c r="A112" s="6" t="str">
-        <x:v>Disc (DKWDRV)</x:v>
+        <x:v>Disabled</x:v>
       </x:c>
       <x:c r="B112" s="7" t="str"/>
       <x:c r="C112" s="5" t="str"/>
       <x:c r="D112" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:2001; bin/POPSLDR/ui.lua:5781; bin/POPSLDR/ui.lua:5810</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5044</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="46" customHeight="1">
       <x:c r="A113" s="6" t="str">
-        <x:v>Discard &amp; Exit</x:v>
+        <x:v>Disc (DKWDRV)</x:v>
       </x:c>
       <x:c r="B113" s="7" t="str"/>
       <x:c r="C113" s="5" t="str"/>
       <x:c r="D113" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:2226</x:v>
+        <x:v>bin/POPSLDR/ui.lua:2001; bin/POPSLDR/ui.lua:5781; bin/POPSLDR/ui.lua:5810</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="46" customHeight="1">
       <x:c r="A114" s="6" t="str">
-        <x:v>Display</x:v>
+        <x:v>Discard &amp; Exit</x:v>
       </x:c>
       <x:c r="B114" s="7" t="str"/>
       <x:c r="C114" s="5" t="str"/>
       <x:c r="D114" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4908</x:v>
+        <x:v>bin/POPSLDR/ui.lua:2226</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="46" customHeight="1">
       <x:c r="A115" s="6" t="str">
-        <x:v>Display reverted -- new mode wasn't confirmed</x:v>
+        <x:v>Display</x:v>
       </x:c>
       <x:c r="B115" s="7" t="str"/>
       <x:c r="C115" s="5" t="str"/>
       <x:c r="D115" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4535</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4908</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="46" customHeight="1">
       <x:c r="A116" s="6" t="str">
-        <x:v>Dithering</x:v>
+        <x:v>Display reverted -- new mode wasn't confirmed</x:v>
       </x:c>
       <x:c r="B116" s="7" t="str"/>
       <x:c r="C116" s="5" t="str"/>
       <x:c r="D116" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3881</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4535</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="46" customHeight="1">
       <x:c r="A117" s="6" t="str">
-        <x:v>Done</x:v>
+        <x:v>Dithering</x:v>
       </x:c>
       <x:c r="B117" s="7" t="str"/>
       <x:c r="C117" s="5" t="str"/>
       <x:c r="D117" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3129; bin/POPSLDR/ui.lua:3992; bin/POPSLDR/ui.lua:4121</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3881</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="46" customHeight="1">
       <x:c r="A118" s="6" t="str">
-        <x:v>ERROR: HDD is not accessible</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="B118" s="7" t="str"/>
       <x:c r="C118" s="5" t="str"/>
       <x:c r="D118" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8899</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3129; bin/POPSLDR/ui.lua:3992; bin/POPSLDR/ui.lua:4121</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="46" customHeight="1">
       <x:c r="A119" s="6" t="str">
-        <x:v>ERROR: Hardware issue detected\nCheck your HDD, network adapter and connection</x:v>
+        <x:v>ERROR: HDD is not accessible</x:v>
       </x:c>
       <x:c r="B119" s="7" t="str"/>
-      <x:c r="C119" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C119" s="5" t="str"/>
       <x:c r="D119" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8903</x:v>
+        <x:v>bin/POPSLDR/system.lua:8930</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="46" customHeight="1">
       <x:c r="A120" s="6" t="str">
-        <x:v>Edit</x:v>
+        <x:v>ERROR: Hardware issue detected\nCheck your HDD, network adapter and connection</x:v>
       </x:c>
       <x:c r="B120" s="7" t="str"/>
-      <x:c r="C120" s="5" t="str"/>
+      <x:c r="C120" s="5" t="str">
+        <x:v>Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D120" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7297</x:v>
+        <x:v>bin/POPSLDR/system.lua:8934</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="46" customHeight="1">
       <x:c r="A121" s="6" t="str">
-        <x:v>Edit %s</x:v>
+        <x:v>Edit</x:v>
       </x:c>
       <x:c r="B121" s="7" t="str"/>
-      <x:c r="C121" s="5" t="str">
-        <x:v>Keep in order: %s</x:v>
-      </x:c>
+      <x:c r="C121" s="5" t="str"/>
       <x:c r="D121" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7296</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7297</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="46" customHeight="1">
       <x:c r="A122" s="6" t="str">
-        <x:v>Edit DKWDRV Path</x:v>
+        <x:v>Edit %s</x:v>
       </x:c>
       <x:c r="B122" s="7" t="str"/>
-      <x:c r="C122" s="5" t="str"/>
+      <x:c r="C122" s="5" t="str">
+        <x:v>Keep in order: %s</x:v>
+      </x:c>
       <x:c r="D122" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4790</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7296</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="46" customHeight="1">
       <x:c r="A123" s="6" t="str">
-        <x:v>Edit POPStarter Path</x:v>
+        <x:v>Edit DKWDRV Path</x:v>
       </x:c>
       <x:c r="B123" s="7" t="str"/>
       <x:c r="C123" s="5" t="str"/>
       <x:c r="D123" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4781</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4790</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="46" customHeight="1">
       <x:c r="A124" s="6" t="str">
-        <x:v>Edit Path</x:v>
+        <x:v>Edit POPStarter Path</x:v>
       </x:c>
       <x:c r="B124" s="7" t="str"/>
       <x:c r="C124" s="5" t="str"/>
       <x:c r="D124" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:2513</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4781</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="46" customHeight="1">
       <x:c r="A125" s="6" t="str">
-        <x:v>Ember 480p requires compatible video output</x:v>
+        <x:v>Edit Path</x:v>
       </x:c>
       <x:c r="B125" s="7" t="str"/>
       <x:c r="C125" s="5" t="str"/>
       <x:c r="D125" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5212</x:v>
+        <x:v>bin/POPSLDR/ui.lua:2513</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="46" customHeight="1">
       <x:c r="A126" s="6" t="str">
-        <x:v>Ember Controller</x:v>
+        <x:v>Ember 480p requires compatible video output</x:v>
       </x:c>
       <x:c r="B126" s="7" t="str"/>
       <x:c r="C126" s="5" t="str"/>
       <x:c r="D126" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5190</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5212</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="46" customHeight="1">
       <x:c r="A127" s="6" t="str">
-        <x:v>Ember Display</x:v>
+        <x:v>Ember Controller</x:v>
       </x:c>
       <x:c r="B127" s="7" t="str"/>
       <x:c r="C127" s="5" t="str"/>
       <x:c r="D127" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5186</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5190</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="46" customHeight="1">
       <x:c r="A128" s="6" t="str">
-        <x:v>Ember Dithering</x:v>
+        <x:v>Ember Display</x:v>
       </x:c>
       <x:c r="B128" s="7" t="str"/>
       <x:c r="C128" s="5" t="str"/>
       <x:c r="D128" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5188</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5186</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="46" customHeight="1">
       <x:c r="A129" s="6" t="str">
-        <x:v>Ember ELF returned: %s</x:v>
+        <x:v>Ember Dithering</x:v>
       </x:c>
       <x:c r="B129" s="7" t="str"/>
-      <x:c r="C129" s="5" t="str">
-        <x:v>Keep in order: %s</x:v>
-      </x:c>
+      <x:c r="C129" s="5" t="str"/>
       <x:c r="D129" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8253</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5188</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="46" customHeight="1">
       <x:c r="A130" s="6" t="str">
-        <x:v>Ember Game Settings</x:v>
+        <x:v>Ember ELF returned: %s</x:v>
       </x:c>
       <x:c r="B130" s="7" t="str"/>
-      <x:c r="C130" s="5" t="str"/>
+      <x:c r="C130" s="5" t="str">
+        <x:v>Keep in order: %s</x:v>
+      </x:c>
       <x:c r="D130" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3912</x:v>
+        <x:v>bin/POPSLDR/system.lua:8266</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="46" customHeight="1">
       <x:c r="A131" s="6" t="str">
-        <x:v>Ember PS1 Core</x:v>
+        <x:v>Ember Game Settings</x:v>
       </x:c>
       <x:c r="B131" s="7" t="str"/>
       <x:c r="C131" s="5" t="str"/>
       <x:c r="D131" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5181</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3912</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="46" customHeight="1">
       <x:c r="A132" s="6" t="str">
-        <x:v>Ember Shading</x:v>
+        <x:v>Ember PS1 Core</x:v>
       </x:c>
       <x:c r="B132" s="7" t="str"/>
       <x:c r="C132" s="5" t="str"/>
       <x:c r="D132" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5189</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5181</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="46" customHeight="1">
       <x:c r="A133" s="6" t="str">
-        <x:v>Ember Timing</x:v>
+        <x:v>Ember Shading</x:v>
       </x:c>
       <x:c r="B133" s="7" t="str"/>
       <x:c r="C133" s="5" t="str"/>
       <x:c r="D133" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5187</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5189</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="46" customHeight="1">
       <x:c r="A134" s="6" t="str">
-        <x:v>Ember did not launch</x:v>
+        <x:v>Ember Timing</x:v>
       </x:c>
       <x:c r="B134" s="7" t="str"/>
       <x:c r="C134" s="5" t="str"/>
       <x:c r="D134" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3694</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5187</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="46" customHeight="1">
       <x:c r="A135" s="6" t="str">
-        <x:v>Ember game scan unavailable</x:v>
+        <x:v>Ember did not launch</x:v>
       </x:c>
       <x:c r="B135" s="7" t="str"/>
       <x:c r="C135" s="5" t="str"/>
       <x:c r="D135" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3130</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3694</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="46" customHeight="1">
       <x:c r="A136" s="6" t="str">
-        <x:v>Ember global settings could not be saved on %s</x:v>
+        <x:v>Ember game scan unavailable</x:v>
       </x:c>
       <x:c r="B136" s="7" t="str"/>
-      <x:c r="C136" s="5" t="str">
-        <x:v>Keep in order: %s</x:v>
-      </x:c>
+      <x:c r="C136" s="5" t="str"/>
       <x:c r="D136" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8233</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3130</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="46" customHeight="1">
       <x:c r="A137" s="6" t="str">
-        <x:v>Ember launch error: %s</x:v>
+        <x:v>Ember global settings could not be saved on %s</x:v>
       </x:c>
       <x:c r="B137" s="7" t="str"/>
       <x:c r="C137" s="5" t="str">
         <x:v>Keep in order: %s</x:v>
       </x:c>
       <x:c r="D137" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8252</x:v>
+        <x:v>bin/POPSLDR/system.lua:8246</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="46" customHeight="1">
       <x:c r="A138" s="6" t="str">
-        <x:v>Ember needs a 512 KB BIOS: %s</x:v>
+        <x:v>Ember launch error: %s</x:v>
       </x:c>
       <x:c r="B138" s="7" t="str"/>
       <x:c r="C138" s="5" t="str">
         <x:v>Keep in order: %s</x:v>
       </x:c>
       <x:c r="D138" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8223</x:v>
+        <x:v>bin/POPSLDR/system.lua:8265</x:v>
       </x:c>
     </x:row>
     <x:row r="139" ht="46" customHeight="1">
       <x:c r="A139" s="6" t="str">
-        <x:v>Enable the POPSTARTER Folder first\n(BDMA / SMB modules must live on the memory card)</x:v>
+        <x:v>Ember needs a 512 KB BIOS: %s</x:v>
       </x:c>
       <x:c r="B139" s="7" t="str"/>
       <x:c r="C139" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
+        <x:v>Keep in order: %s</x:v>
       </x:c>
       <x:c r="D139" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4871; bin/POPSLDR/ui.lua:4895</x:v>
+        <x:v>bin/POPSLDR/system.lua:8236</x:v>
       </x:c>
     </x:row>
     <x:row r="140" ht="46" customHeight="1">
       <x:c r="A140" s="6" t="str">
-        <x:v>Enable the POPSTARTER Folder first\n(SMB modules must live on the memory card)</x:v>
+        <x:v>Enable the POPSTARTER Folder first\n(BDMA / SMB modules must live on the memory card)</x:v>
       </x:c>
       <x:c r="B140" s="7" t="str"/>
       <x:c r="C140" s="5" t="str">
         <x:v>Keep literal \n line breaks</x:v>
       </x:c>
       <x:c r="D140" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7326</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4871; bin/POPSLDR/ui.lua:4895</x:v>
       </x:c>
     </x:row>
     <x:row r="141" ht="46" customHeight="1">
       <x:c r="A141" s="6" t="str">
-        <x:v>Enter</x:v>
+        <x:v>Enable the POPSTARTER Folder first\n(SMB modules must live on the memory card)</x:v>
       </x:c>
       <x:c r="B141" s="7" t="str"/>
-      <x:c r="C141" s="5" t="str"/>
+      <x:c r="C141" s="5" t="str">
+        <x:v>Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D141" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:1466</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7326</x:v>
       </x:c>
     </x:row>
     <x:row r="142" ht="46" customHeight="1">
       <x:c r="A142" s="6" t="str">
-        <x:v>Ethernet protocol</x:v>
+        <x:v>Enter</x:v>
       </x:c>
       <x:c r="B142" s="7" t="str"/>
       <x:c r="C142" s="5" t="str"/>
       <x:c r="D142" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7108</x:v>
+        <x:v>bin/POPSLDR/ui.lua:1466</x:v>
       </x:c>
     </x:row>
     <x:row r="143" ht="46" customHeight="1">
       <x:c r="A143" s="6" t="str">
-        <x:v>Exit</x:v>
+        <x:v>Ethernet protocol</x:v>
       </x:c>
       <x:c r="B143" s="7" t="str"/>
       <x:c r="C143" s="5" t="str"/>
       <x:c r="D143" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:1460; bin/POPSLDR/ui.lua:1991</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7108</x:v>
       </x:c>
     </x:row>
     <x:row r="144" ht="46" customHeight="1">
       <x:c r="A144" s="6" t="str">
-        <x:v>FAT32-USB (None)</x:v>
+        <x:v>Exit</x:v>
       </x:c>
       <x:c r="B144" s="7" t="str"/>
       <x:c r="C144" s="5" t="str"/>
       <x:c r="D144" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:1178</x:v>
+        <x:v>bin/POPSLDR/ui.lua:1460; bin/POPSLDR/ui.lua:1991</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="46" customHeight="1">
       <x:c r="A145" s="6" t="str">
-        <x:v>Failed to apply FAT32 BDMA</x:v>
+        <x:v>FAT32-USB (None)</x:v>
       </x:c>
       <x:c r="B145" s="7" t="str"/>
       <x:c r="C145" s="5" t="str"/>
       <x:c r="D145" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:7074</x:v>
+        <x:v>bin/POPSLDR/ui.lua:1178</x:v>
       </x:c>
     </x:row>
     <x:row r="146" ht="46" customHeight="1">
       <x:c r="A146" s="6" t="str">
-        <x:v>Failed to connect to SMB</x:v>
+        <x:v>Failed to apply FAT32 BDMA</x:v>
       </x:c>
       <x:c r="B146" s="7" t="str"/>
       <x:c r="C146" s="5" t="str"/>
       <x:c r="D146" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7040</x:v>
+        <x:v>bin/POPSLDR/system.lua:7074</x:v>
       </x:c>
     </x:row>
     <x:row r="147" ht="46" customHeight="1">
       <x:c r="A147" s="6" t="str">
-        <x:v>Failed to install SMB modules</x:v>
+        <x:v>Failed to connect to SMB</x:v>
       </x:c>
       <x:c r="B147" s="7" t="str"/>
       <x:c r="C147" s="5" t="str"/>
       <x:c r="D147" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6977</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7040</x:v>
       </x:c>
     </x:row>
     <x:row r="148" ht="46" customHeight="1">
       <x:c r="A148" s="6" t="str">
-        <x:v>Failed to load HDD</x:v>
+        <x:v>Failed to install SMB modules</x:v>
       </x:c>
       <x:c r="B148" s="7" t="str"/>
       <x:c r="C148" s="5" t="str"/>
       <x:c r="D148" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:9212; bin/POPSLDR/ui.lua:6224</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6977</x:v>
       </x:c>
     </x:row>
     <x:row r="149" ht="46" customHeight="1">
       <x:c r="A149" s="6" t="str">
-        <x:v>Failed to load HDD (exFAT)</x:v>
+        <x:v>Failed to load HDD</x:v>
       </x:c>
       <x:c r="B149" s="7" t="str"/>
       <x:c r="C149" s="5" t="str"/>
       <x:c r="D149" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6167</x:v>
+        <x:v>bin/POPSLDR/system.lua:9243; bin/POPSLDR/ui.lua:6224</x:v>
       </x:c>
     </x:row>
     <x:row r="150" ht="46" customHeight="1">
       <x:c r="A150" s="6" t="str">
-        <x:v>Failed to load MMCE</x:v>
+        <x:v>Failed to load HDD (exFAT)</x:v>
       </x:c>
       <x:c r="B150" s="7" t="str"/>
       <x:c r="C150" s="5" t="str"/>
       <x:c r="D150" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6065</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6167</x:v>
       </x:c>
     </x:row>
     <x:row r="151" ht="46" customHeight="1">
       <x:c r="A151" s="6" t="str">
-        <x:v>Failed to load MX4SIO</x:v>
+        <x:v>Failed to load MMCE</x:v>
       </x:c>
       <x:c r="B151" s="7" t="str"/>
       <x:c r="C151" s="5" t="str"/>
       <x:c r="D151" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6107</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6065</x:v>
       </x:c>
     </x:row>
     <x:row r="152" ht="46" customHeight="1">
       <x:c r="A152" s="6" t="str">
-        <x:v>Failed to load USB</x:v>
+        <x:v>Failed to load MX4SIO</x:v>
       </x:c>
       <x:c r="B152" s="7" t="str"/>
       <x:c r="C152" s="5" t="str"/>
       <x:c r="D152" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6301</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6107</x:v>
       </x:c>
     </x:row>
     <x:row r="153" ht="46" customHeight="1">
       <x:c r="A153" s="6" t="str">
-        <x:v>Failed to refresh HDD list</x:v>
+        <x:v>Failed to load USB</x:v>
       </x:c>
       <x:c r="B153" s="7" t="str"/>
       <x:c r="C153" s="5" t="str"/>
       <x:c r="D153" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3993</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6301</x:v>
       </x:c>
     </x:row>
     <x:row r="154" ht="46" customHeight="1">
       <x:c r="A154" s="6" t="str">
-        <x:v>Failed to refresh list</x:v>
+        <x:v>Failed to refresh HDD list</x:v>
       </x:c>
       <x:c r="B154" s="7" t="str"/>
       <x:c r="C154" s="5" t="str"/>
       <x:c r="D154" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4122</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3993</x:v>
       </x:c>
     </x:row>
     <x:row r="155" ht="46" customHeight="1">
       <x:c r="A155" s="6" t="str">
-        <x:v>Failed to remove some SMB modules</x:v>
+        <x:v>Failed to refresh list</x:v>
       </x:c>
       <x:c r="B155" s="7" t="str"/>
       <x:c r="C155" s="5" t="str"/>
       <x:c r="D155" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:7558</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4122</x:v>
       </x:c>
     </x:row>
     <x:row r="156" ht="46" customHeight="1">
       <x:c r="A156" s="6" t="str">
-        <x:v>Failed to save settings</x:v>
+        <x:v>Failed to remove some SMB modules</x:v>
       </x:c>
       <x:c r="B156" s="7" t="str"/>
       <x:c r="C156" s="5" t="str"/>
       <x:c r="D156" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:5410</x:v>
+        <x:v>bin/POPSLDR/system.lua:7571</x:v>
       </x:c>
     </x:row>
     <x:row r="157" ht="46" customHeight="1">
       <x:c r="A157" s="6" t="str">
-        <x:v>Finalizing settings</x:v>
+        <x:v>Failed to save settings</x:v>
       </x:c>
       <x:c r="B157" s="7" t="str"/>
       <x:c r="C157" s="5" t="str"/>
       <x:c r="D157" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:5970</x:v>
+        <x:v>bin/POPSLDR/system.lua:5410</x:v>
       </x:c>
     </x:row>
     <x:row r="158" ht="46" customHeight="1">
       <x:c r="A158" s="6" t="str">
-        <x:v>First disc only</x:v>
+        <x:v>Finalizing settings</x:v>
       </x:c>
       <x:c r="B158" s="7" t="str"/>
       <x:c r="C158" s="5" t="str"/>
       <x:c r="D158" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5063</x:v>
+        <x:v>bin/POPSLDR/system.lua:5970</x:v>
       </x:c>
     </x:row>
     <x:row r="159" ht="46" customHeight="1">
       <x:c r="A159" s="6" t="str">
-        <x:v>Game List</x:v>
+        <x:v>First disc only</x:v>
       </x:c>
       <x:c r="B159" s="7" t="str"/>
       <x:c r="C159" s="5" t="str"/>
       <x:c r="D159" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5060</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5063</x:v>
       </x:c>
     </x:row>
     <x:row r="160" ht="46" customHeight="1">
       <x:c r="A160" s="6" t="str">
-        <x:v>Game details</x:v>
+        <x:v>Game List</x:v>
       </x:c>
       <x:c r="B160" s="7" t="str"/>
       <x:c r="C160" s="5" t="str"/>
       <x:c r="D160" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5094</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5060</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="46" customHeight="1">
       <x:c r="A161" s="6" t="str">
-        <x:v>Game file missing</x:v>
+        <x:v>Game details</x:v>
       </x:c>
       <x:c r="B161" s="7" t="str"/>
       <x:c r="C161" s="5" t="str"/>
       <x:c r="D161" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3837</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5094</x:v>
       </x:c>
     </x:row>
     <x:row r="162" ht="46" customHeight="1">
       <x:c r="A162" s="6" t="str">
-        <x:v>Game hidden</x:v>
+        <x:v>Game file missing</x:v>
       </x:c>
       <x:c r="B162" s="7" t="str"/>
       <x:c r="C162" s="5" t="str"/>
       <x:c r="D162" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4157; bin/POPSLDR/ui.lua:4175</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3837</x:v>
       </x:c>
     </x:row>
     <x:row r="163" ht="46" customHeight="1">
       <x:c r="A163" s="6" t="str">
-        <x:v>Game list cache</x:v>
+        <x:v>Game hidden</x:v>
       </x:c>
       <x:c r="B163" s="7" t="str"/>
       <x:c r="C163" s="5" t="str"/>
       <x:c r="D163" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5115</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4157; bin/POPSLDR/ui.lua:4175</x:v>
       </x:c>
     </x:row>
     <x:row r="164" ht="46" customHeight="1">
       <x:c r="A164" s="6" t="str">
-        <x:v>Game shown</x:v>
+        <x:v>Game list cache</x:v>
       </x:c>
       <x:c r="B164" s="7" t="str"/>
       <x:c r="C164" s="5" t="str"/>
       <x:c r="D164" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4157; bin/POPSLDR/ui.lua:4175</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5115</x:v>
       </x:c>
     </x:row>
     <x:row r="165" ht="46" customHeight="1">
       <x:c r="A165" s="6" t="str">
-        <x:v>GameName derivation failed</x:v>
+        <x:v>Game shown</x:v>
       </x:c>
       <x:c r="B165" s="7" t="str"/>
       <x:c r="C165" s="5" t="str"/>
       <x:c r="D165" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10109</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4157; bin/POPSLDR/ui.lua:4175</x:v>
       </x:c>
     </x:row>
     <x:row r="166" ht="46" customHeight="1">
       <x:c r="A166" s="6" t="str">
-        <x:v>Games path (folder holding POPS)</x:v>
+        <x:v>GameName derivation failed</x:v>
       </x:c>
       <x:c r="B166" s="7" t="str"/>
       <x:c r="C166" s="5" t="str"/>
       <x:c r="D166" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7214</x:v>
+        <x:v>bin/POPSLDR/system.lua:10140</x:v>
       </x:c>
     </x:row>
     <x:row r="167" ht="46" customHeight="1">
       <x:c r="A167" s="6" t="str">
-        <x:v>Games path affects browsing only:\nPOPStarter can only launch games from &lt;share&gt;/POPS</x:v>
+        <x:v>Games path (folder holding POPS)</x:v>
       </x:c>
       <x:c r="B167" s="7" t="str"/>
-      <x:c r="C167" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C167" s="5" t="str"/>
       <x:c r="D167" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7027</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7214</x:v>
       </x:c>
     </x:row>
     <x:row r="168" ht="46" customHeight="1">
       <x:c r="A168" s="6" t="str">
-        <x:v>Games will list but will not boot\nInstall them from Settings &gt; SMB modules when ready</x:v>
+        <x:v>Games path affects browsing only:\nPOPStarter can only launch games from &lt;share&gt;/POPS</x:v>
       </x:c>
       <x:c r="B168" s="7" t="str"/>
       <x:c r="C168" s="5" t="str">
         <x:v>Keep literal \n line breaks</x:v>
       </x:c>
       <x:c r="D168" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6986</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7027</x:v>
       </x:c>
     </x:row>
     <x:row r="169" ht="46" customHeight="1">
       <x:c r="A169" s="6" t="str">
-        <x:v>Gateway</x:v>
+        <x:v>Games will list but will not boot\nInstall them from Settings &gt; SMB modules when ready</x:v>
       </x:c>
       <x:c r="B169" s="7" t="str"/>
-      <x:c r="C169" s="5" t="str"/>
+      <x:c r="C169" s="5" t="str">
+        <x:v>Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D169" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7211</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6986</x:v>
       </x:c>
     </x:row>
     <x:row r="170" ht="46" customHeight="1">
       <x:c r="A170" s="6" t="str">
-        <x:v>HDD (exFAT)</x:v>
+        <x:v>Gateway</x:v>
       </x:c>
       <x:c r="B170" s="7" t="str"/>
       <x:c r="C170" s="5" t="str"/>
       <x:c r="D170" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3013; bin/POPSLDR/ui.lua:5781; bin/POPSLDR/ui.lua:5805</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7211</x:v>
       </x:c>
     </x:row>
     <x:row r="171" ht="46" customHeight="1">
       <x:c r="A171" s="6" t="str">
-        <x:v>HDD Alt</x:v>
+        <x:v>HDD (exFAT)</x:v>
       </x:c>
       <x:c r="B171" s="7" t="str"/>
       <x:c r="C171" s="5" t="str"/>
       <x:c r="D171" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4226</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3013; bin/POPSLDR/ui.lua:5781; bin/POPSLDR/ui.lua:5805</x:v>
       </x:c>
     </x:row>
     <x:row r="172" ht="46" customHeight="1">
       <x:c r="A172" s="6" t="str">
-        <x:v>HDD Alt mode needs POPSTARTER on HDD</x:v>
+        <x:v>HDD Alt</x:v>
       </x:c>
       <x:c r="B172" s="7" t="str"/>
       <x:c r="C172" s="5" t="str"/>
       <x:c r="D172" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3777</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4226</x:v>
       </x:c>
     </x:row>
     <x:row r="173" ht="46" customHeight="1">
       <x:c r="A173" s="6" t="str">
-        <x:v>HDD boot mount lost during settings write\nReboot to restore HDD access</x:v>
+        <x:v>HDD Alt mode needs POPSTARTER on HDD</x:v>
       </x:c>
       <x:c r="B173" s="7" t="str"/>
-      <x:c r="C173" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C173" s="5" t="str"/>
       <x:c r="D173" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:2351</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3777</x:v>
       </x:c>
     </x:row>
     <x:row r="174" ht="46" customHeight="1">
       <x:c r="A174" s="6" t="str">
-        <x:v>HDD dir read failed:</x:v>
+        <x:v>HDD boot mount lost during settings write\nReboot to restore HDD access</x:v>
       </x:c>
       <x:c r="B174" s="7" t="str"/>
-      <x:c r="C174" s="5" t="str"/>
+      <x:c r="C174" s="5" t="str">
+        <x:v>Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D174" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8577</x:v>
+        <x:v>bin/POPSLDR/system.lua:2351</x:v>
       </x:c>
     </x:row>
     <x:row r="175" ht="46" customHeight="1">
       <x:c r="A175" s="6" t="str">
-        <x:v>HDD game-partition write test FAILED (%s)</x:v>
+        <x:v>HDD dir read failed:</x:v>
       </x:c>
       <x:c r="B175" s="7" t="str"/>
-      <x:c r="C175" s="5" t="str">
-        <x:v>Keep in order: %s</x:v>
-      </x:c>
+      <x:c r="C175" s="5" t="str"/>
       <x:c r="D175" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4513</x:v>
+        <x:v>bin/POPSLDR/system.lua:8608</x:v>
       </x:c>
     </x:row>
     <x:row r="176" ht="46" customHeight="1">
       <x:c r="A176" s="6" t="str">
-        <x:v>HDD is ready now (status recovered)</x:v>
+        <x:v>HDD game-partition write test FAILED (%s)</x:v>
       </x:c>
       <x:c r="B176" s="7" t="str"/>
-      <x:c r="C176" s="5" t="str"/>
+      <x:c r="C176" s="5" t="str">
+        <x:v>Keep in order: %s</x:v>
+      </x:c>
       <x:c r="D176" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8918</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4513</x:v>
       </x:c>
     </x:row>
     <x:row r="177" ht="46" customHeight="1">
       <x:c r="A177" s="6" t="str">
-        <x:v>HDD list loaded from cache (R1 rescans)</x:v>
+        <x:v>HDD is ready now (status recovered)</x:v>
       </x:c>
       <x:c r="B177" s="7" t="str"/>
       <x:c r="C177" s="5" t="str"/>
       <x:c r="D177" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6183</x:v>
+        <x:v>bin/POPSLDR/system.lua:8949</x:v>
       </x:c>
     </x:row>
     <x:row r="178" ht="46" customHeight="1">
       <x:c r="A178" s="6" t="str">
-        <x:v>HDD list refreshed</x:v>
+        <x:v>HDD list loaded from cache (R1 rescans)</x:v>
       </x:c>
       <x:c r="B178" s="7" t="str"/>
       <x:c r="C178" s="5" t="str"/>
       <x:c r="D178" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4024</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6183</x:v>
       </x:c>
     </x:row>
     <x:row r="179" ht="46" customHeight="1">
       <x:c r="A179" s="6" t="str">
-        <x:v>HDD list refreshed (no games found)</x:v>
+        <x:v>HDD list refreshed</x:v>
       </x:c>
       <x:c r="B179" s="7" t="str"/>
       <x:c r="C179" s="5" t="str"/>
       <x:c r="D179" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4022</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4024</x:v>
       </x:c>
     </x:row>
     <x:row r="180" ht="46" customHeight="1">
       <x:c r="A180" s="6" t="str">
-        <x:v>HDD modules not loaded</x:v>
+        <x:v>HDD list refreshed (no games found)</x:v>
       </x:c>
       <x:c r="B180" s="7" t="str"/>
       <x:c r="C180" s="5" t="str"/>
       <x:c r="D180" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:987</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4022</x:v>
       </x:c>
     </x:row>
     <x:row r="181" ht="46" customHeight="1">
       <x:c r="A181" s="6" t="str">
-        <x:v>HDD not usable</x:v>
+        <x:v>HDD modules not loaded</x:v>
       </x:c>
       <x:c r="B181" s="7" t="str"/>
       <x:c r="C181" s="5" t="str"/>
       <x:c r="D181" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6220</x:v>
+        <x:v>bin/POPSLDR/system.lua:987</x:v>
       </x:c>
     </x:row>
     <x:row r="182" ht="46" customHeight="1">
       <x:c r="A182" s="6" t="str">
-        <x:v>Hidden</x:v>
+        <x:v>HDD not usable</x:v>
       </x:c>
       <x:c r="B182" s="7" t="str"/>
       <x:c r="C182" s="5" t="str"/>
       <x:c r="D182" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5025; bin/POPSLDR/ui.lua:5070</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6220</x:v>
       </x:c>
     </x:row>
     <x:row r="183" ht="46" customHeight="1">
       <x:c r="A183" s="6" t="str">
-        <x:v>Hidden games</x:v>
+        <x:v>Hidden</x:v>
       </x:c>
       <x:c r="B183" s="7" t="str"/>
       <x:c r="C183" s="5" t="str"/>
       <x:c r="D183" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5069</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5025; bin/POPSLDR/ui.lua:5070</x:v>
       </x:c>
     </x:row>
     <x:row r="184" ht="46" customHeight="1">
       <x:c r="A184" s="6" t="str">
-        <x:v>Hidden games are already shown here (dimmed)\nEnable "Hide hidden games" in Settings to filter them out</x:v>
+        <x:v>Hidden games</x:v>
       </x:c>
       <x:c r="B184" s="7" t="str"/>
-      <x:c r="C184" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C184" s="5" t="str"/>
       <x:c r="D184" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:3950</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5069</x:v>
       </x:c>
     </x:row>
     <x:row r="185" ht="46" customHeight="1">
       <x:c r="A185" s="6" t="str">
-        <x:v>Hidden games are filtered out.\nPress R3 to reveal them, then L3 to unhide.</x:v>
+        <x:v>Hidden games are already shown here (dimmed)\nEnable "Hide hidden games" in Settings to filter them out</x:v>
       </x:c>
       <x:c r="B185" s="7" t="str"/>
       <x:c r="C185" s="5" t="str">
         <x:v>Keep literal \n line breaks</x:v>
       </x:c>
       <x:c r="D185" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4151</x:v>
+        <x:v>bin/POPSLDR/ui.lua:3950</x:v>
       </x:c>
     </x:row>
     <x:row r="186" ht="46" customHeight="1">
       <x:c r="A186" s="6" t="str">
-        <x:v>Hidden games filtered out again</x:v>
+        <x:v>Hidden games are filtered out.\nPress R3 to reveal them, then L3 to unhide.</x:v>
       </x:c>
       <x:c r="B186" s="7" t="str"/>
-      <x:c r="C186" s="5" t="str"/>
+      <x:c r="C186" s="5" t="str">
+        <x:v>Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D186" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4209</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4151</x:v>
       </x:c>
     </x:row>
     <x:row r="187" ht="46" customHeight="1">
       <x:c r="A187" s="6" t="str">
-        <x:v>Hide UI Text</x:v>
+        <x:v>Hidden games filtered out again</x:v>
       </x:c>
       <x:c r="B187" s="7" t="str"/>
       <x:c r="C187" s="5" t="str"/>
       <x:c r="D187" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4944</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4209</x:v>
       </x:c>
     </x:row>
     <x:row r="188" ht="46" customHeight="1">
       <x:c r="A188" s="6" t="str">
-        <x:v>How to hide a game</x:v>
+        <x:v>Hide UI Text</x:v>
       </x:c>
       <x:c r="B188" s="7" t="str"/>
       <x:c r="C188" s="5" t="str"/>
       <x:c r="D188" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5080</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4944</x:v>
       </x:c>
     </x:row>
     <x:row r="189" ht="46" customHeight="1">
       <x:c r="A189" s="6" t="str">
-        <x:v>IP address</x:v>
+        <x:v>How to hide a game</x:v>
       </x:c>
       <x:c r="B189" s="7" t="str"/>
       <x:c r="C189" s="5" t="str"/>
       <x:c r="D189" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7218</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5080</x:v>
       </x:c>
     </x:row>
     <x:row r="190" ht="46" customHeight="1">
       <x:c r="A190" s="6" t="str">
-        <x:v>IP assignment</x:v>
+        <x:v>IP address</x:v>
       </x:c>
       <x:c r="B190" s="7" t="str"/>
       <x:c r="C190" s="5" t="str"/>
       <x:c r="D190" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7210</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7218</x:v>
       </x:c>
     </x:row>
     <x:row r="191" ht="46" customHeight="1">
       <x:c r="A191" s="6" t="str">
-        <x:v>Initializing UDPFS network filesystem...</x:v>
+        <x:v>IP assignment</x:v>
       </x:c>
       <x:c r="B191" s="7" t="str"/>
       <x:c r="C191" s="5" t="str"/>
       <x:c r="D191" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8399</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7210</x:v>
       </x:c>
     </x:row>
     <x:row r="192" ht="46" customHeight="1">
       <x:c r="A192" s="6" t="str">
-        <x:v>Initializing USB backend...</x:v>
+        <x:v>Initializing UDPFS network filesystem...</x:v>
       </x:c>
       <x:c r="B192" s="7" t="str"/>
       <x:c r="C192" s="5" t="str"/>
       <x:c r="D192" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4109; bin/POPSLDR/ui.lua:6230</x:v>
+        <x:v>bin/POPSLDR/system.lua:8412</x:v>
       </x:c>
     </x:row>
     <x:row r="193" ht="46" customHeight="1">
       <x:c r="A193" s="6" t="str">
-        <x:v>Install them now?</x:v>
+        <x:v>Initializing USB backend...</x:v>
       </x:c>
       <x:c r="B193" s="7" t="str"/>
       <x:c r="C193" s="5" t="str"/>
       <x:c r="D193" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6969</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4109; bin/POPSLDR/ui.lua:6230</x:v>
       </x:c>
     </x:row>
     <x:row r="194" ht="46" customHeight="1">
       <x:c r="A194" s="6" t="str">
-        <x:v>Installed</x:v>
+        <x:v>Install them now?</x:v>
       </x:c>
       <x:c r="B194" s="7" t="str"/>
       <x:c r="C194" s="5" t="str"/>
       <x:c r="D194" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5150</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6969</x:v>
       </x:c>
     </x:row>
     <x:row r="195" ht="46" customHeight="1">
       <x:c r="A195" s="6" t="str">
-        <x:v>Installing SMB modules...</x:v>
+        <x:v>Installed</x:v>
       </x:c>
       <x:c r="B195" s="7" t="str"/>
       <x:c r="C195" s="5" t="str"/>
       <x:c r="D195" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6973</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5150</x:v>
       </x:c>
     </x:row>
     <x:row r="196" ht="46" customHeight="1">
       <x:c r="A196" s="6" t="str">
-        <x:v>Internal HDD</x:v>
+        <x:v>Installing SMB modules...</x:v>
       </x:c>
       <x:c r="B196" s="7" t="str"/>
       <x:c r="C196" s="5" t="str"/>
       <x:c r="D196" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5053</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6973</x:v>
       </x:c>
     </x:row>
     <x:row r="197" ht="46" customHeight="1">
       <x:c r="A197" s="6" t="str">
-        <x:v>Internal error: game_base derived as POPSTARTER; refusing to launch.</x:v>
+        <x:v>Internal HDD</x:v>
       </x:c>
       <x:c r="B197" s="7" t="str"/>
       <x:c r="C197" s="5" t="str"/>
       <x:c r="D197" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10184</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5053</x:v>
       </x:c>
     </x:row>
     <x:row r="198" ht="46" customHeight="1">
       <x:c r="A198" s="6" t="str">
-        <x:v>Invalid Ember game selection</x:v>
+        <x:v>Internal error: game_base derived as POPSTARTER; refusing to launch.</x:v>
       </x:c>
       <x:c r="B198" s="7" t="str"/>
       <x:c r="C198" s="5" t="str"/>
       <x:c r="D198" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8207</x:v>
+        <x:v>bin/POPSLDR/system.lua:10215</x:v>
       </x:c>
     </x:row>
     <x:row r="199" ht="46" customHeight="1">
       <x:c r="A199" s="6" t="str">
-        <x:v>Invalid HDD game entry</x:v>
+        <x:v>Invalid Ember game selection</x:v>
       </x:c>
       <x:c r="B199" s="7" t="str"/>
       <x:c r="C199" s="5" t="str"/>
       <x:c r="D199" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10057</x:v>
+        <x:v>bin/POPSLDR/system.lua:8220</x:v>
       </x:c>
     </x:row>
     <x:row r="200" ht="46" customHeight="1">
       <x:c r="A200" s="6" t="str">
-        <x:v>Invalid game selection</x:v>
+        <x:v>Invalid HDD game entry</x:v>
       </x:c>
       <x:c r="B200" s="7" t="str"/>
       <x:c r="C200" s="5" t="str"/>
       <x:c r="D200" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:9981</x:v>
+        <x:v>bin/POPSLDR/system.lua:10088</x:v>
       </x:c>
     </x:row>
     <x:row r="201" ht="46" customHeight="1">
       <x:c r="A201" s="6" t="str">
-        <x:v>Keep</x:v>
+        <x:v>Invalid game selection</x:v>
       </x:c>
       <x:c r="B201" s="7" t="str"/>
       <x:c r="C201" s="5" t="str"/>
       <x:c r="D201" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7153</x:v>
+        <x:v>bin/POPSLDR/system.lua:10012</x:v>
       </x:c>
     </x:row>
     <x:row r="202" ht="46" customHeight="1">
       <x:c r="A202" s="6" t="str">
-        <x:v>Keep this display mode?</x:v>
+        <x:v>Keep</x:v>
       </x:c>
       <x:c r="B202" s="7" t="str"/>
       <x:c r="C202" s="5" t="str"/>
       <x:c r="D202" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7152</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7153</x:v>
       </x:c>
     </x:row>
     <x:row r="203" ht="46" customHeight="1">
       <x:c r="A203" s="6" t="str">
-        <x:v>Keep-IOP ELF loader unavailable</x:v>
+        <x:v>Keep this display mode?</x:v>
       </x:c>
       <x:c r="B203" s="7" t="str"/>
       <x:c r="C203" s="5" t="str"/>
       <x:c r="D203" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8209</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7152</x:v>
       </x:c>
     </x:row>
     <x:row r="204" ht="46" customHeight="1">
       <x:c r="A204" s="6" t="str">
-        <x:v>Keyboard Layout</x:v>
+        <x:v>Keep-IOP ELF loader unavailable</x:v>
       </x:c>
       <x:c r="B204" s="7" t="str"/>
       <x:c r="C204" s="5" t="str"/>
       <x:c r="D204" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4975</x:v>
+        <x:v>bin/POPSLDR/system.lua:8222</x:v>
       </x:c>
     </x:row>
     <x:row r="205" ht="46" customHeight="1">
       <x:c r="A205" s="6" t="str">
-        <x:v>L3 on the game list</x:v>
+        <x:v>Keyboard Layout</x:v>
       </x:c>
       <x:c r="B205" s="7" t="str"/>
       <x:c r="C205" s="5" t="str"/>
       <x:c r="D205" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5081</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4975</x:v>
       </x:c>
     </x:row>
     <x:row r="206" ht="46" customHeight="1">
       <x:c r="A206" s="6" t="str">
-        <x:v>LAUNCH FAILED</x:v>
+        <x:v>L3 on the game list</x:v>
       </x:c>
       <x:c r="B206" s="7" t="str"/>
       <x:c r="C206" s="5" t="str"/>
       <x:c r="D206" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:9599</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5081</x:v>
       </x:c>
     </x:row>
     <x:row r="207" ht="46" customHeight="1">
       <x:c r="A207" s="6" t="str">
-        <x:v>Language</x:v>
+        <x:v>LAUNCH FAILED</x:v>
       </x:c>
       <x:c r="B207" s="7" t="str"/>
       <x:c r="C207" s="5" t="str"/>
       <x:c r="D207" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4983</x:v>
+        <x:v>bin/POPSLDR/system.lua:9630</x:v>
       </x:c>
     </x:row>
     <x:row r="208" ht="46" customHeight="1">
       <x:c r="A208" s="6" t="str">
-        <x:v>Launch</x:v>
+        <x:v>Language</x:v>
       </x:c>
       <x:c r="B208" s="7" t="str"/>
       <x:c r="C208" s="5" t="str"/>
       <x:c r="D208" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:1468</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4983</x:v>
       </x:c>
     </x:row>
     <x:row r="209" ht="46" customHeight="1">
       <x:c r="A209" s="6" t="str">
-        <x:v>Launch DKWDRV?</x:v>
+        <x:v>Launch</x:v>
       </x:c>
       <x:c r="B209" s="7" t="str"/>
       <x:c r="C209" s="5" t="str"/>
       <x:c r="D209" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:2002</x:v>
+        <x:v>bin/POPSLDR/ui.lua:1468</x:v>
       </x:c>
     </x:row>
     <x:row r="210" ht="46" customHeight="1">
       <x:c r="A210" s="6" t="str">
-        <x:v>Left aligned</x:v>
+        <x:v>Launch DKWDRV?</x:v>
       </x:c>
       <x:c r="B210" s="7" t="str"/>
       <x:c r="C210" s="5" t="str"/>
       <x:c r="D210" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5084</x:v>
+        <x:v>bin/POPSLDR/ui.lua:2002</x:v>
       </x:c>
     </x:row>
     <x:row r="211" ht="46" customHeight="1">
       <x:c r="A211" s="6" t="str">
-        <x:v>Link mode</x:v>
+        <x:v>Left aligned</x:v>
       </x:c>
       <x:c r="B211" s="7" t="str"/>
       <x:c r="C211" s="5" t="str"/>
       <x:c r="D211" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7211</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5084</x:v>
       </x:c>
     </x:row>
     <x:row r="212" ht="46" customHeight="1">
       <x:c r="A212" s="6" t="str">
-        <x:v>List refreshed</x:v>
+        <x:v>Link mode</x:v>
       </x:c>
       <x:c r="B212" s="7" t="str"/>
       <x:c r="C212" s="5" t="str"/>
       <x:c r="D212" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4133</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7211</x:v>
       </x:c>
     </x:row>
     <x:row r="213" ht="46" customHeight="1">
       <x:c r="A213" s="6" t="str">
-        <x:v>List refreshed (no games found)</x:v>
+        <x:v>List refreshed</x:v>
       </x:c>
       <x:c r="B213" s="7" t="str"/>
       <x:c r="C213" s="5" t="str"/>
       <x:c r="D213" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4131</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4133</x:v>
       </x:c>
     </x:row>
     <x:row r="214" ht="46" customHeight="1">
       <x:c r="A214" s="6" t="str">
-        <x:v>Loaded MMCE list from cache...</x:v>
+        <x:v>List refreshed (no games found)</x:v>
       </x:c>
       <x:c r="B214" s="7" t="str"/>
       <x:c r="C214" s="5" t="str"/>
       <x:c r="D214" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6055</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4131</x:v>
       </x:c>
     </x:row>
     <x:row r="215" ht="46" customHeight="1">
       <x:c r="A215" s="6" t="str">
-        <x:v>Loaded MX4SIO list from cache...</x:v>
+        <x:v>Loaded MMCE list from cache...</x:v>
       </x:c>
       <x:c r="B215" s="7" t="str"/>
       <x:c r="C215" s="5" t="str"/>
       <x:c r="D215" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6099</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6055</x:v>
       </x:c>
     </x:row>
     <x:row r="216" ht="46" customHeight="1">
       <x:c r="A216" s="6" t="str">
-        <x:v>Loaded SMB list from cache...</x:v>
+        <x:v>Loaded MX4SIO list from cache...</x:v>
       </x:c>
       <x:c r="B216" s="7" t="str"/>
       <x:c r="C216" s="5" t="str"/>
       <x:c r="D216" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7013</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6099</x:v>
       </x:c>
     </x:row>
     <x:row r="217" ht="46" customHeight="1">
       <x:c r="A217" s="6" t="str">
-        <x:v>Loaded USB list from cache...</x:v>
+        <x:v>Loaded SMB list from cache...</x:v>
       </x:c>
       <x:c r="B217" s="7" t="str"/>
       <x:c r="C217" s="5" t="str"/>
       <x:c r="D217" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6282</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7013</x:v>
       </x:c>
     </x:row>
     <x:row r="218" ht="46" customHeight="1">
       <x:c r="A218" s="6" t="str">
-        <x:v>Loaded exFAT HDD list from cache...</x:v>
+        <x:v>Loaded USB list from cache...</x:v>
       </x:c>
       <x:c r="B218" s="7" t="str"/>
       <x:c r="C218" s="5" t="str"/>
       <x:c r="D218" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6159</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6282</x:v>
       </x:c>
     </x:row>
     <x:row r="219" ht="46" customHeight="1">
       <x:c r="A219" s="6" t="str">
-        <x:v>Loading HDD (exFAT)...</x:v>
+        <x:v>Loaded exFAT HDD list from cache...</x:v>
       </x:c>
       <x:c r="B219" s="7" t="str"/>
       <x:c r="C219" s="5" t="str"/>
       <x:c r="D219" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6110</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6159</x:v>
       </x:c>
     </x:row>
     <x:row r="220" ht="46" customHeight="1">
       <x:c r="A220" s="6" t="str">
-        <x:v>Loading HDD modules...</x:v>
+        <x:v>Loading HDD (exFAT)...</x:v>
       </x:c>
       <x:c r="B220" s="7" t="str"/>
       <x:c r="C220" s="5" t="str"/>
       <x:c r="D220" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6173</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6110</x:v>
       </x:c>
     </x:row>
     <x:row r="221" ht="46" customHeight="1">
       <x:c r="A221" s="6" t="str">
-        <x:v>Loading HDD...</x:v>
+        <x:v>Loading HDD modules...</x:v>
       </x:c>
       <x:c r="B221" s="7" t="str"/>
       <x:c r="C221" s="5" t="str"/>
       <x:c r="D221" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6170</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6173</x:v>
       </x:c>
     </x:row>
     <x:row r="222" ht="46" customHeight="1">
       <x:c r="A222" s="6" t="str">
-        <x:v>Loading MMCE...</x:v>
+        <x:v>Loading HDD...</x:v>
       </x:c>
       <x:c r="B222" s="7" t="str"/>
       <x:c r="C222" s="5" t="str"/>
       <x:c r="D222" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6019</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6170</x:v>
       </x:c>
     </x:row>
     <x:row r="223" ht="46" customHeight="1">
       <x:c r="A223" s="6" t="str">
-        <x:v>Loading MX4SIO...</x:v>
+        <x:v>Loading MMCE...</x:v>
       </x:c>
       <x:c r="B223" s="7" t="str"/>
       <x:c r="C223" s="5" t="str"/>
       <x:c r="D223" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6068</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6019</x:v>
       </x:c>
     </x:row>
     <x:row r="224" ht="46" customHeight="1">
       <x:c r="A224" s="6" t="str">
-        <x:v>Loading UDPFS network drivers...</x:v>
+        <x:v>Loading MX4SIO...</x:v>
       </x:c>
       <x:c r="B224" s="7" t="str"/>
       <x:c r="C224" s="5" t="str"/>
       <x:c r="D224" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7088</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6068</x:v>
       </x:c>
     </x:row>
     <x:row r="225" ht="46" customHeight="1">
       <x:c r="A225" s="6" t="str">
-        <x:v>Loading USB...</x:v>
+        <x:v>Loading UDPFS network drivers...</x:v>
       </x:c>
       <x:c r="B225" s="7" t="str"/>
       <x:c r="C225" s="5" t="str"/>
       <x:c r="D225" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6227</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7088</x:v>
       </x:c>
     </x:row>
     <x:row r="226" ht="46" customHeight="1">
       <x:c r="A226" s="6" t="str">
-        <x:v>Loading network modules...</x:v>
+        <x:v>Loading USB...</x:v>
       </x:c>
       <x:c r="B226" s="7" t="str"/>
       <x:c r="C226" s="5" t="str"/>
       <x:c r="D226" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8457</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6227</x:v>
       </x:c>
     </x:row>
     <x:row r="227" ht="46" customHeight="1">
       <x:c r="A227" s="6" t="str">
-        <x:v>Locating MX4SIO POPS folder...</x:v>
+        <x:v>Loading network modules...</x:v>
       </x:c>
       <x:c r="B227" s="7" t="str"/>
       <x:c r="C227" s="5" t="str"/>
       <x:c r="D227" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6076</x:v>
+        <x:v>bin/POPSLDR/system.lua:8488</x:v>
       </x:c>
     </x:row>
     <x:row r="228" ht="46" customHeight="1">
       <x:c r="A228" s="6" t="str">
-        <x:v>Locating exFAT HDD POPS folder...</x:v>
+        <x:v>Locating MX4SIO POPS folder...</x:v>
       </x:c>
       <x:c r="B228" s="7" t="str"/>
       <x:c r="C228" s="5" t="str"/>
       <x:c r="D228" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6122</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6076</x:v>
       </x:c>
     </x:row>
     <x:row r="229" ht="46" customHeight="1">
       <x:c r="A229" s="6" t="str">
-        <x:v>Logging on to the share...</x:v>
+        <x:v>Locating exFAT HDD POPS folder...</x:v>
       </x:c>
       <x:c r="B229" s="7" t="str"/>
       <x:c r="C229" s="5" t="str"/>
       <x:c r="D229" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8473</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6122</x:v>
       </x:c>
     </x:row>
     <x:row r="230" ht="46" customHeight="1">
       <x:c r="A230" s="6" t="str">
-        <x:v>Looking for USB drive...</x:v>
+        <x:v>Logging on to the share...</x:v>
       </x:c>
       <x:c r="B230" s="7" t="str"/>
       <x:c r="C230" s="5" t="str"/>
       <x:c r="D230" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6243</x:v>
+        <x:v>bin/POPSLDR/system.lua:8504</x:v>
       </x:c>
     </x:row>
     <x:row r="231" ht="46" customHeight="1">
       <x:c r="A231" s="6" t="str">
-        <x:v>MMCE has no POPS folder\nexpected mmce0:/POPS/</x:v>
+        <x:v>Looking for USB drive...</x:v>
       </x:c>
       <x:c r="B231" s="7" t="str"/>
-      <x:c r="C231" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C231" s="5" t="str"/>
       <x:c r="D231" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6061</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6243</x:v>
       </x:c>
     </x:row>
     <x:row r="232" ht="46" customHeight="1">
       <x:c r="A232" s="6" t="str">
-        <x:v>MX4SIO driver failed to load\ntry the page again, or reboot</x:v>
+        <x:v>MMCE has no POPS folder\nexpected mmce0:/POPS/</x:v>
       </x:c>
       <x:c r="B232" s="7" t="str"/>
       <x:c r="C232" s="5" t="str">
         <x:v>Keep literal \n line breaks</x:v>
       </x:c>
       <x:c r="D232" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6085</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6061</x:v>
       </x:c>
     </x:row>
     <x:row r="233" ht="46" customHeight="1">
       <x:c r="A233" s="6" t="str">
-        <x:v>Memory Card</x:v>
+        <x:v>MX4SIO driver failed to load\ntry the page again, or reboot</x:v>
       </x:c>
       <x:c r="B233" s="7" t="str"/>
-      <x:c r="C233" s="5" t="str"/>
+      <x:c r="C233" s="5" t="str">
+        <x:v>Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D233" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5349</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6085</x:v>
       </x:c>
     </x:row>
     <x:row r="234" ht="46" customHeight="1">
       <x:c r="A234" s="6" t="str">
-        <x:v>Menu</x:v>
+        <x:v>Memory Card</x:v>
       </x:c>
       <x:c r="B234" s="7" t="str"/>
       <x:c r="C234" s="5" t="str"/>
       <x:c r="D234" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:1463</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5349</x:v>
       </x:c>
     </x:row>
     <x:row r="235" ht="46" customHeight="1">
       <x:c r="A235" s="6" t="str">
-        <x:v>Missing %s</x:v>
+        <x:v>Menu</x:v>
       </x:c>
       <x:c r="B235" s="7" t="str"/>
-      <x:c r="C235" s="5" t="str">
-        <x:v>Keep in order: %s</x:v>
-      </x:c>
+      <x:c r="C235" s="5" t="str"/>
       <x:c r="D235" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8220</x:v>
+        <x:v>bin/POPSLDR/ui.lua:1463</x:v>
       </x:c>
     </x:row>
     <x:row r="236" ht="46" customHeight="1">
       <x:c r="A236" s="6" t="str">
-        <x:v>Missing %s -- UDPFS requires the POPS folder on each USB volume</x:v>
+        <x:v>Missing %s</x:v>
       </x:c>
       <x:c r="B236" s="7" t="str"/>
       <x:c r="C236" s="5" t="str">
         <x:v>Keep in order: %s</x:v>
       </x:c>
       <x:c r="D236" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8426</x:v>
+        <x:v>bin/POPSLDR/system.lua:8233</x:v>
       </x:c>
     </x:row>
     <x:row r="237" ht="46" customHeight="1">
@@ -2790,7 +2790,7 @@
       <x:c r="B237" s="7" t="str"/>
       <x:c r="C237" s="5" t="str"/>
       <x:c r="D237" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:7717</x:v>
+        <x:v>bin/POPSLDR/system.lua:7730</x:v>
       </x:c>
     </x:row>
     <x:row r="238" ht="46" customHeight="1">
@@ -2800,7 +2800,7 @@
       <x:c r="B238" s="7" t="str"/>
       <x:c r="C238" s="5" t="str"/>
       <x:c r="D238" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:7111; bin/POPSLDR/system.lua:7152</x:v>
+        <x:v>bin/POPSLDR/system.lua:7115; bin/POPSLDR/system.lua:7157</x:v>
       </x:c>
     </x:row>
     <x:row r="239" ht="46" customHeight="1">
@@ -2810,7 +2810,7 @@
       <x:c r="B239" s="7" t="str"/>
       <x:c r="C239" s="5" t="str"/>
       <x:c r="D239" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:7473</x:v>
+        <x:v>bin/POPSLDR/system.lua:7486</x:v>
       </x:c>
     </x:row>
     <x:row r="240" ht="46" customHeight="1">
@@ -2916,7 +2916,7 @@
         <x:v>Keep in order: %s</x:v>
       </x:c>
       <x:c r="D249" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8227</x:v>
+        <x:v>bin/POPSLDR/system.lua:8240</x:v>
       </x:c>
     </x:row>
     <x:row r="250" ht="46" customHeight="1">
@@ -2961,7 +2961,7 @@
         <x:v>bin/POPSLDR/ui.lua:3764</x:v>
       </x:c>
     </x:row>
-    <x:row r="254" ht="61" customHeight="1">
+    <x:row r="254" ht="46" customHeight="1">
       <x:c r="A254" s="6" t="str">
         <x:v>No POPSTARTER.ELF found\nPOPSTARTER is never read from the share -- put it in mc0:/POPSTARTER/,\nor beside POPSLOADER.ELF, or set Settings &gt; POPSTARTER Path</x:v>
       </x:c>
@@ -3028,7 +3028,7 @@
         <x:v>Keep literal \n line breaks</x:v>
       </x:c>
       <x:c r="D259" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10461; bin/POPSLDR/ui.lua:6150</x:v>
+        <x:v>bin/POPSLDR/system.lua:10492; bin/POPSLDR/ui.lua:6150</x:v>
       </x:c>
     </x:row>
     <x:row r="260" ht="46" customHeight="1">
@@ -3217,22 +3217,22 @@
     </x:row>
     <x:row r="278" ht="46" customHeight="1">
       <x:c r="A278" s="6" t="str">
-        <x:v>Opening USB list...</x:v>
+        <x:v>Opening UDPFS...</x:v>
       </x:c>
       <x:c r="B278" s="7" t="str"/>
       <x:c r="C278" s="5" t="str"/>
       <x:c r="D278" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6299</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7086</x:v>
       </x:c>
     </x:row>
     <x:row r="279" ht="46" customHeight="1">
       <x:c r="A279" s="6" t="str">
-        <x:v>Opening USB+UDPFS...</x:v>
+        <x:v>Opening USB list...</x:v>
       </x:c>
       <x:c r="B279" s="7" t="str"/>
       <x:c r="C279" s="5" t="str"/>
       <x:c r="D279" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7086</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6299</x:v>
       </x:c>
     </x:row>
     <x:row r="280" ht="46" customHeight="1">
@@ -3418,7 +3418,7 @@
         <x:v>Keep in order: %s, %s</x:v>
       </x:c>
       <x:c r="D297" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:9596</x:v>
+        <x:v>bin/POPSLDR/system.lua:9627</x:v>
       </x:c>
     </x:row>
     <x:row r="298" ht="46" customHeight="1">
@@ -3518,7 +3518,7 @@
       <x:c r="B307" s="7" t="str"/>
       <x:c r="C307" s="5" t="str"/>
       <x:c r="D307" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10459; bin/POPSLDR/ui.lua:6148</x:v>
+        <x:v>bin/POPSLDR/system.lua:10490; bin/POPSLDR/ui.lua:6148</x:v>
       </x:c>
     </x:row>
     <x:row r="308" ht="46" customHeight="1">
@@ -3645,12 +3645,10 @@
     </x:row>
     <x:row r="320" ht="46" customHeight="1">
       <x:c r="A320" s="6" t="str">
-        <x:v>SMB already owns the network adapter\nRestart POPSLoader to switch to USB+UDPFS</x:v>
+        <x:v>SMB already owns the network adapter\nRestart POPSLoader to switch to UDPFS</x:v>
       </x:c>
       <x:c r="B320" s="7" t="str"/>
-      <x:c r="C320" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C320" s="5" t="str"/>
       <x:c r="D320" s="5" t="str">
         <x:v>bin/POPSLDR/ui.lua:6930</x:v>
       </x:c>
@@ -3972,7 +3970,7 @@
       <x:c r="B351" s="7" t="str"/>
       <x:c r="C351" s="5" t="str"/>
       <x:c r="D351" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8387</x:v>
+        <x:v>bin/POPSLDR/system.lua:8400</x:v>
       </x:c>
     </x:row>
     <x:row r="352" ht="46" customHeight="1">
@@ -4074,7 +4072,7 @@
       <x:c r="B361" s="7" t="str"/>
       <x:c r="C361" s="5" t="str"/>
       <x:c r="D361" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10146</x:v>
+        <x:v>bin/POPSLDR/system.lua:10177</x:v>
       </x:c>
     </x:row>
     <x:row r="362" ht="46" customHeight="1">
@@ -4084,7 +4082,7 @@
       <x:c r="B362" s="7" t="str"/>
       <x:c r="C362" s="5" t="str"/>
       <x:c r="D362" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:7258</x:v>
+        <x:v>bin/POPSLDR/system.lua:7271</x:v>
       </x:c>
     </x:row>
     <x:row r="363" ht="46" customHeight="1">
@@ -4096,7 +4094,7 @@
         <x:v>Keep literal \n line breaks</x:v>
       </x:c>
       <x:c r="D363" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10828</x:v>
+        <x:v>bin/POPSLDR/system.lua:10859</x:v>
       </x:c>
     </x:row>
     <x:row r="364" ht="46" customHeight="1">
@@ -4116,7 +4114,7 @@
       <x:c r="B365" s="7" t="str"/>
       <x:c r="C365" s="5" t="str"/>
       <x:c r="D365" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:7264; bin/POPSLDR/ui.lua:3853</x:v>
+        <x:v>bin/POPSLDR/system.lua:7277; bin/POPSLDR/ui.lua:3853</x:v>
       </x:c>
     </x:row>
     <x:row r="366" ht="46" customHeight="1">
@@ -4170,7 +4168,7 @@
         <x:v>Keep literal \n line breaks</x:v>
       </x:c>
       <x:c r="D370" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8878; bin/POPSLDR/ui.lua:6141</x:v>
+        <x:v>bin/POPSLDR/system.lua:8909; bin/POPSLDR/ui.lua:6141</x:v>
       </x:c>
     </x:row>
     <x:row r="371" ht="46" customHeight="1">
@@ -4195,7 +4193,7 @@
         <x:v>bin/POPSLDR/ui.lua:3161; bin/POPSLDR/ui.lua:6304</x:v>
       </x:c>
     </x:row>
-    <x:row r="373" ht="61" customHeight="1">
+    <x:row r="373" ht="46" customHeight="1">
       <x:c r="A373" s="6" t="str">
         <x:v>This removes the POPSTARTER pack -- including the\nBDMA and SMB modules -- from mc0: / mc1:. They won't\nreturn until you turn this back On (or re-add them\nmanually). Your POPSLoader settings are kept.</x:v>
       </x:c>
@@ -4229,424 +4227,436 @@
     </x:row>
     <x:row r="376" ht="46" customHeight="1">
       <x:c r="A376" s="6" t="str">
-        <x:v>UDPFS IP changed after network initialization\nRestart POPSLoader to apply the new static PS2 IP</x:v>
+        <x:v>UDPFS (network R/W)</x:v>
       </x:c>
       <x:c r="B376" s="7" t="str"/>
-      <x:c r="C376" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C376" s="5" t="str"/>
       <x:c r="D376" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6929</x:v>
+        <x:v>bin/POPSLDR/ui.lua:1183</x:v>
       </x:c>
     </x:row>
     <x:row r="377" ht="46" customHeight="1">
       <x:c r="A377" s="6" t="str">
-        <x:v>UDPFS SMAP driver failed to load</x:v>
+        <x:v>UDPFS IP changed after network initialization\nRestart POPSLoader to apply the new static PS2 IP</x:v>
       </x:c>
       <x:c r="B377" s="7" t="str"/>
-      <x:c r="C377" s="5" t="str"/>
+      <x:c r="C377" s="5" t="str">
+        <x:v>Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D377" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6932</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6929</x:v>
       </x:c>
     </x:row>
     <x:row r="378" ht="46" customHeight="1">
       <x:c r="A378" s="6" t="str">
-        <x:v>UDPFS USB IPCONFIG.DAT conflicts with the menu settings:\n%s\nEdit it to match %s %s (not overwritten)</x:v>
+        <x:v>UDPFS IPCONFIG.DAT conflicts with menu settings:\n%s\nEdit it to match %s %s (not overwritten)</x:v>
       </x:c>
       <x:c r="B378" s="7" t="str"/>
       <x:c r="C378" s="5" t="str">
-        <x:v>Keep in order: %s, %s, %s; Keep literal \n line breaks</x:v>
+        <x:v>Keep in order: %s; %s; %s</x:v>
       </x:c>
       <x:c r="D378" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8435</x:v>
+        <x:v>bin/POPSLDR/system.lua:8451</x:v>
       </x:c>
     </x:row>
     <x:row r="379" ht="46" customHeight="1">
       <x:c r="A379" s="6" t="str">
-        <x:v>UDPFS already owns the network adapter.\nRestart POPSLoader to switch to SMBv1.</x:v>
+        <x:v>UDPFS SMAP driver failed to load</x:v>
       </x:c>
       <x:c r="B379" s="7" t="str"/>
-      <x:c r="C379" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C379" s="5" t="str"/>
       <x:c r="D379" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7113</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6932</x:v>
       </x:c>
     </x:row>
     <x:row r="380" ht="46" customHeight="1">
       <x:c r="A380" s="6" t="str">
-        <x:v>UDPFS driver staging failed -- launch cancelled</x:v>
+        <x:v>UDPFS already owns the network adapter.\nRestart POPSLoader to switch to SMBv1.</x:v>
       </x:c>
       <x:c r="B380" s="7" t="str"/>
-      <x:c r="C380" s="5" t="str"/>
+      <x:c r="C380" s="5" t="str">
+        <x:v>Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D380" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10150</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7113</x:v>
       </x:c>
     </x:row>
     <x:row r="381" ht="46" customHeight="1">
       <x:c r="A381" s="6" t="str">
-        <x:v>UDPFS filesystem module failed to load</x:v>
+        <x:v>UDPFS config must contain 1-120 bytes:\n%s</x:v>
       </x:c>
       <x:c r="B381" s="7" t="str"/>
-      <x:c r="C381" s="5" t="str"/>
+      <x:c r="C381" s="5" t="str">
+        <x:v>Keep in order: %s</x:v>
+      </x:c>
       <x:c r="D381" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6934</x:v>
+        <x:v>bin/POPSLDR/system.lua:8463</x:v>
       </x:c>
     </x:row>
     <x:row r="382" ht="46" customHeight="1">
       <x:c r="A382" s="6" t="str">
-        <x:v>UDPFS menu modules are not available</x:v>
+        <x:v>UDPFS driver staging failed -- launch cancelled</x:v>
       </x:c>
       <x:c r="B382" s="7" t="str"/>
       <x:c r="C382" s="5" t="str"/>
       <x:c r="D382" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8397</x:v>
+        <x:v>bin/POPSLDR/system.lua:10181</x:v>
       </x:c>
     </x:row>
     <x:row r="383" ht="46" customHeight="1">
       <x:c r="A383" s="6" t="str">
-        <x:v>UDPFS module initialization failed</x:v>
+        <x:v>UDPFS filesystem module failed to load</x:v>
       </x:c>
       <x:c r="B383" s="7" t="str"/>
       <x:c r="C383" s="5" t="str"/>
       <x:c r="D383" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8401</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6934</x:v>
       </x:c>
     </x:row>
     <x:row r="384" ht="46" customHeight="1">
       <x:c r="A384" s="6" t="str">
-        <x:v>UDPFS needs a static PS2 address. Turn off DHCP in Settings &gt; SMB / Network.</x:v>
+        <x:v>UDPFS menu modules are not available</x:v>
       </x:c>
       <x:c r="B384" s="7" t="str"/>
       <x:c r="C384" s="5" t="str"/>
       <x:c r="D384" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8378</x:v>
+        <x:v>bin/POPSLDR/system.lua:8410</x:v>
       </x:c>
     </x:row>
     <x:row r="385" ht="46" customHeight="1">
       <x:c r="A385" s="6" t="str">
-        <x:v>UDPFS network initialization incomplete\nRestart POPSLoader</x:v>
+        <x:v>UDPFS menu support is missing from this build</x:v>
       </x:c>
       <x:c r="B385" s="7" t="str"/>
-      <x:c r="C385" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C385" s="5" t="str"/>
       <x:c r="D385" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6931</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7073</x:v>
       </x:c>
     </x:row>
     <x:row r="386" ht="46" customHeight="1">
       <x:c r="A386" s="6" t="str">
-        <x:v>UDPFS network stack failed to load</x:v>
+        <x:v>UDPFS module initialization failed</x:v>
       </x:c>
       <x:c r="B386" s="7" t="str"/>
       <x:c r="C386" s="5" t="str"/>
       <x:c r="D386" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6933</x:v>
+        <x:v>bin/POPSLDR/system.lua:8414</x:v>
       </x:c>
     </x:row>
     <x:row r="387" ht="46" customHeight="1">
       <x:c r="A387" s="6" t="str">
-        <x:v>UDPFS server unavailable\nCheck your network and UDPFS server</x:v>
+        <x:v>UDPFS needs a static PS2 address. Turn off DHCP in Settings &gt; SMB / Network.</x:v>
       </x:c>
       <x:c r="B387" s="7" t="str"/>
-      <x:c r="C387" s="5" t="str">
-        <x:v>Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C387" s="5" t="str"/>
       <x:c r="D387" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:6928</x:v>
+        <x:v>bin/POPSLDR/system.lua:8391</x:v>
       </x:c>
     </x:row>
     <x:row r="388" ht="46" customHeight="1">
       <x:c r="A388" s="6" t="str">
-        <x:v>UI text hidden</x:v>
+        <x:v>UDPFS network initialization incomplete\nRestart POPSLoader</x:v>
       </x:c>
       <x:c r="B388" s="7" t="str"/>
-      <x:c r="C388" s="5" t="str"/>
+      <x:c r="C388" s="5" t="str">
+        <x:v>Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D388" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:1240</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6931</x:v>
       </x:c>
     </x:row>
     <x:row r="389" ht="46" customHeight="1">
       <x:c r="A389" s="6" t="str">
-        <x:v>UI text shown</x:v>
+        <x:v>UDPFS network stack failed to load</x:v>
       </x:c>
       <x:c r="B389" s="7" t="str"/>
       <x:c r="C389" s="5" t="str"/>
       <x:c r="D389" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:1242</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6933</x:v>
       </x:c>
     </x:row>
     <x:row r="390" ht="46" customHeight="1">
       <x:c r="A390" s="6" t="str">
-        <x:v>USB+UDPFS menu support is missing from this build</x:v>
+        <x:v>UDPFS requires POPSTARTER modules on a memory card</x:v>
       </x:c>
       <x:c r="B390" s="7" t="str"/>
       <x:c r="C390" s="5" t="str"/>
       <x:c r="D390" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7073</x:v>
+        <x:v>bin/POPSLDR/system.lua:10169</x:v>
       </x:c>
     </x:row>
     <x:row r="391" ht="46" customHeight="1">
       <x:c r="A391" s="6" t="str">
-        <x:v>USB+UDPFS requires POPSTARTER modules on a memory card</x:v>
+        <x:v>UDPFS server unavailable\nCheck your network and UDPFS server</x:v>
       </x:c>
       <x:c r="B391" s="7" t="str"/>
-      <x:c r="C391" s="5" t="str"/>
+      <x:c r="C391" s="5" t="str">
+        <x:v>Keep literal \n line breaks</x:v>
+      </x:c>
       <x:c r="D391" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:10138</x:v>
+        <x:v>bin/POPSLDR/ui.lua:6928</x:v>
       </x:c>
     </x:row>
     <x:row r="392" ht="46" customHeight="1">
       <x:c r="A392" s="6" t="str">
-        <x:v>USB+UDPFS requires a USB volume with POPS/ installed</x:v>
+        <x:v>UDPFS: %s\nCheck the static PS2 IP, cable and UDPFS server</x:v>
       </x:c>
       <x:c r="B392" s="7" t="str"/>
-      <x:c r="C392" s="5" t="str"/>
+      <x:c r="C392" s="5" t="str">
+        <x:v>Keep in order: %s</x:v>
+      </x:c>
       <x:c r="D392" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8418</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7091</x:v>
       </x:c>
     </x:row>
     <x:row r="393" ht="46" customHeight="1">
       <x:c r="A393" s="6" t="str">
-        <x:v>USB+UDPFS: %s\nCheck the static PS2 IP, cable and UDPFS server</x:v>
+        <x:v>UI text hidden</x:v>
       </x:c>
       <x:c r="B393" s="7" t="str"/>
-      <x:c r="C393" s="5" t="str">
-        <x:v>Keep in order: %s; Keep literal \n line breaks</x:v>
-      </x:c>
+      <x:c r="C393" s="5" t="str"/>
       <x:c r="D393" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7091</x:v>
+        <x:v>bin/POPSLDR/ui.lua:1240</x:v>
       </x:c>
     </x:row>
     <x:row r="394" ht="46" customHeight="1">
       <x:c r="A394" s="6" t="str">
-        <x:v>Unable to keep Ember PFS mount</x:v>
+        <x:v>UI text shown</x:v>
       </x:c>
       <x:c r="B394" s="7" t="str"/>
       <x:c r="C394" s="5" t="str"/>
       <x:c r="D394" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8243</x:v>
+        <x:v>bin/POPSLDR/ui.lua:1242</x:v>
       </x:c>
     </x:row>
     <x:row r="395" ht="46" customHeight="1">
       <x:c r="A395" s="6" t="str">
-        <x:v>Unchanged</x:v>
+        <x:v>Unable to keep Ember PFS mount</x:v>
       </x:c>
       <x:c r="B395" s="7" t="str"/>
-      <x:c r="C395" s="5" t="str">
-        <x:v>Ember: Unchanged preserves a setting; Default removes the override</x:v>
-      </x:c>
+      <x:c r="C395" s="5" t="str"/>
       <x:c r="D395" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5218</x:v>
+        <x:v>bin/POPSLDR/system.lua:8256</x:v>
       </x:c>
     </x:row>
     <x:row r="396" ht="46" customHeight="1">
       <x:c r="A396" s="6" t="str">
-        <x:v>Unknown BDMA mode:</x:v>
+        <x:v>Unchanged</x:v>
       </x:c>
       <x:c r="B396" s="7" t="str"/>
-      <x:c r="C396" s="5" t="str"/>
+      <x:c r="C396" s="5" t="str">
+        <x:v>Ember: Unchanged preserves a setting; Default removes the override</x:v>
+      </x:c>
       <x:c r="D396" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:7090</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5218</x:v>
       </x:c>
     </x:row>
     <x:row r="397" ht="46" customHeight="1">
       <x:c r="A397" s="6" t="str">
-        <x:v>User</x:v>
+        <x:v>Unknown BDMA mode:</x:v>
       </x:c>
       <x:c r="B397" s="7" t="str"/>
       <x:c r="C397" s="5" t="str"/>
       <x:c r="D397" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7213</x:v>
+        <x:v>bin/POPSLDR/system.lua:7092</x:v>
       </x:c>
     </x:row>
     <x:row r="398" ht="46" customHeight="1">
       <x:c r="A398" s="6" t="str">
-        <x:v>Version</x:v>
+        <x:v>User</x:v>
       </x:c>
       <x:c r="B398" s="7" t="str"/>
       <x:c r="C398" s="5" t="str"/>
       <x:c r="D398" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5370</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7213</x:v>
       </x:c>
     </x:row>
     <x:row r="399" ht="46" customHeight="1">
       <x:c r="A399" s="6" t="str">
-        <x:v>Video Standard</x:v>
+        <x:v>Version</x:v>
       </x:c>
       <x:c r="B399" s="7" t="str"/>
       <x:c r="C399" s="5" t="str"/>
       <x:c r="D399" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4910</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5370</x:v>
       </x:c>
     </x:row>
     <x:row r="400" ht="46" customHeight="1">
       <x:c r="A400" s="6" t="str">
-        <x:v>Visible (manage)</x:v>
+        <x:v>Video Standard</x:v>
       </x:c>
       <x:c r="B400" s="7" t="str"/>
       <x:c r="C400" s="5" t="str"/>
       <x:c r="D400" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:5070</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4910</x:v>
       </x:c>
     </x:row>
     <x:row r="401" ht="46" customHeight="1">
       <x:c r="A401" s="6" t="str">
-        <x:v>WARNING: HDD has no APA format</x:v>
+        <x:v>Visible (manage)</x:v>
       </x:c>
       <x:c r="B401" s="7" t="str"/>
       <x:c r="C401" s="5" t="str"/>
       <x:c r="D401" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8897</x:v>
+        <x:v>bin/POPSLDR/ui.lua:5070</x:v>
       </x:c>
     </x:row>
     <x:row r="402" ht="46" customHeight="1">
       <x:c r="A402" s="6" t="str">
-        <x:v>WARNING: No HDD detected</x:v>
+        <x:v>WARNING: HDD has no APA format</x:v>
       </x:c>
       <x:c r="B402" s="7" t="str"/>
       <x:c r="C402" s="5" t="str"/>
       <x:c r="D402" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8901</x:v>
+        <x:v>bin/POPSLDR/system.lua:8928</x:v>
       </x:c>
     </x:row>
     <x:row r="403" ht="46" customHeight="1">
       <x:c r="A403" s="6" t="str">
-        <x:v>Waiting for link + DHCP lease...</x:v>
+        <x:v>WARNING: No HDD detected</x:v>
       </x:c>
       <x:c r="B403" s="7" t="str"/>
       <x:c r="C403" s="5" t="str"/>
       <x:c r="D403" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8467</x:v>
+        <x:v>bin/POPSLDR/system.lua:8932</x:v>
       </x:c>
     </x:row>
     <x:row r="404" ht="46" customHeight="1">
       <x:c r="A404" s="6" t="str">
-        <x:v>Waiting for network link...</x:v>
+        <x:v>Waiting for link + DHCP lease...</x:v>
       </x:c>
       <x:c r="B404" s="7" t="str"/>
       <x:c r="C404" s="5" t="str"/>
       <x:c r="D404" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:8467</x:v>
+        <x:v>bin/POPSLDR/system.lua:8498</x:v>
       </x:c>
     </x:row>
     <x:row r="405" ht="46" customHeight="1">
       <x:c r="A405" s="6" t="str">
-        <x:v>Working...</x:v>
+        <x:v>Waiting for network link...</x:v>
       </x:c>
       <x:c r="B405" s="7" t="str"/>
       <x:c r="C405" s="5" t="str"/>
       <x:c r="D405" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:1303; bin/POPSLDR/ui.lua:1305; bin/POPSLDR/ui.lua:1324</x:v>
+        <x:v>bin/POPSLDR/system.lua:8498</x:v>
       </x:c>
     </x:row>
     <x:row r="406" ht="46" customHeight="1">
       <x:c r="A406" s="6" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Working...</x:v>
       </x:c>
       <x:c r="B406" s="7" t="str"/>
       <x:c r="C406" s="5" t="str"/>
       <x:c r="D406" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:2003; bin/POPSLDR/ui.lua:6845</x:v>
+        <x:v>bin/POPSLDR/ui.lua:1303; bin/POPSLDR/ui.lua:1305; bin/POPSLDR/ui.lua:1324</x:v>
       </x:c>
     </x:row>
     <x:row r="407" ht="46" customHeight="1">
       <x:c r="A407" s="6" t="str">
-        <x:v>You can still add a "&lt;game&gt;.hide" next to the .VCD from a PC.</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="B407" s="7" t="str"/>
       <x:c r="C407" s="5" t="str"/>
       <x:c r="D407" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4167</x:v>
+        <x:v>bin/POPSLDR/ui.lua:2003; bin/POPSLDR/ui.lua:6845</x:v>
       </x:c>
     </x:row>
     <x:row r="408" ht="46" customHeight="1">
       <x:c r="A408" s="6" t="str">
-        <x:v>__.POPS partition %s accepts writes (game-partition RW test)</x:v>
+        <x:v>You can still add a "&lt;game&gt;.hide" next to the .VCD from a PC.</x:v>
       </x:c>
       <x:c r="B408" s="7" t="str"/>
-      <x:c r="C408" s="5" t="str">
-        <x:v>Keep in order: %s</x:v>
-      </x:c>
+      <x:c r="C408" s="5" t="str"/>
       <x:c r="D408" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:4511</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4167</x:v>
       </x:c>
     </x:row>
     <x:row r="409" ht="46" customHeight="1">
       <x:c r="A409" s="6" t="str">
-        <x:v>adjusted -- using</x:v>
+        <x:v>__.POPS partition %s accepts writes (game-partition RW test)</x:v>
       </x:c>
       <x:c r="B409" s="7" t="str"/>
-      <x:c r="C409" s="5" t="str"/>
+      <x:c r="C409" s="5" t="str">
+        <x:v>Keep in order: %s</x:v>
+      </x:c>
       <x:c r="D409" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7313</x:v>
+        <x:v>bin/POPSLDR/ui.lua:4511</x:v>
       </x:c>
     </x:row>
     <x:row r="410" ht="46" customHeight="1">
       <x:c r="A410" s="6" t="str">
-        <x:v>check the memory card, or turn Adaptive BDMA off</x:v>
+        <x:v>adjusted -- using</x:v>
       </x:c>
       <x:c r="B410" s="7" t="str"/>
       <x:c r="C410" s="5" t="str"/>
       <x:c r="D410" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:7272</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7313</x:v>
       </x:c>
     </x:row>
     <x:row r="411" ht="46" customHeight="1">
       <x:c r="A411" s="6" t="str">
-        <x:v>exFAT-HDD (ata)</x:v>
+        <x:v>check the memory card, or turn Adaptive BDMA off</x:v>
       </x:c>
       <x:c r="B411" s="7" t="str"/>
       <x:c r="C411" s="5" t="str"/>
       <x:c r="D411" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:1182</x:v>
+        <x:v>bin/POPSLDR/system.lua:7285</x:v>
       </x:c>
     </x:row>
     <x:row r="412" ht="46" customHeight="1">
       <x:c r="A412" s="6" t="str">
-        <x:v>if not confirmed</x:v>
+        <x:v>exFAT-HDD (ata)</x:v>
       </x:c>
       <x:c r="B412" s="7" t="str"/>
       <x:c r="C412" s="5" t="str"/>
       <x:c r="D412" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:7154</x:v>
+        <x:v>bin/POPSLDR/ui.lua:1182</x:v>
       </x:c>
     </x:row>
     <x:row r="413" ht="46" customHeight="1">
       <x:c r="A413" s="6" t="str">
-        <x:v>re-select it under Settings &gt; Storage to restage</x:v>
+        <x:v>if not confirmed</x:v>
       </x:c>
       <x:c r="B413" s="7" t="str"/>
       <x:c r="C413" s="5" t="str"/>
       <x:c r="D413" s="5" t="str">
-        <x:v>bin/POPSLDR/system.lua:5929</x:v>
+        <x:v>bin/POPSLDR/ui.lua:7154</x:v>
       </x:c>
     </x:row>
     <x:row r="414" ht="46" customHeight="1">
       <x:c r="A414" s="6" t="str">
-        <x:v>return code:</x:v>
+        <x:v>re-select it under Settings &gt; Storage to restage</x:v>
       </x:c>
       <x:c r="B414" s="7" t="str"/>
       <x:c r="C414" s="5" t="str"/>
       <x:c r="D414" s="5" t="str">
-        <x:v>bin/POPSLDR/ui.lua:2205; bin/POPSLDR/ui.lua:2295</x:v>
+        <x:v>bin/POPSLDR/system.lua:5929</x:v>
       </x:c>
     </x:row>
     <x:row r="415" ht="46" customHeight="1">
       <x:c r="A415" s="6" t="str">
-        <x:v>status:</x:v>
+        <x:v>return code:</x:v>
       </x:c>
       <x:c r="B415" s="7" t="str"/>
       <x:c r="C415" s="5" t="str"/>
       <x:c r="D415" s="5" t="str">
+        <x:v>bin/POPSLDR/ui.lua:2205; bin/POPSLDR/ui.lua:2295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="416" ht="46" customHeight="1">
+      <x:c r="A416" s="6" t="str">
+        <x:v>status:</x:v>
+      </x:c>
+      <x:c r="B416" s="7" t="str"/>
+      <x:c r="C416" s="5" t="str"/>
+      <x:c r="D416" s="5" t="str">
         <x:v>bin/POPSLDR/ui.lua:6220</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea3edcaae082448e"/>
+    <x:tablePart ns1:id="Rea3edcaae082448e"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>